<commit_message>
Added protocolRelationships ID code
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/nwss-reporting-to-v2/ids/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{638F6E2D-9375-B04D-AB5F-D9C3F40BFEF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B0AA56B-8624-9448-A1E4-922A9BA6E2B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -265,9 +265,6 @@
     <t>fn.datetimetz(dat.samples.__collDT.split('/!/'))</t>
   </si>
   <si>
-    <t>"pr"</t>
-  </si>
-  <si>
     <t>protocolRelationshipsID</t>
   </si>
   <si>
@@ -320,6 +317,9 @@
   </si>
   <si>
     <t>fn.makeid(datEmpty.qualityReports.qualityFlag, dat.qualityReports.measureRepID, dat.qualityReports.sampleID, dat.qualityReports.measureSetRepID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.protocolRelationships.protocolIDContainer, datEmpty.protocolRelationships.stepIDObj, datEmpty.protocolRelationships.relationshipID)</t>
   </si>
 </sst>
 </file>
@@ -711,7 +711,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D2" t="s">
         <v>74</v>
@@ -739,7 +739,7 @@
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D5" t="s">
         <v>59</v>
@@ -788,10 +788,10 @@
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -834,7 +834,7 @@
         <v>16</v>
       </c>
       <c r="C18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D18" t="s">
         <v>60</v>
@@ -889,7 +889,7 @@
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D25" t="s">
         <v>61</v>
@@ -994,7 +994,7 @@
         <v>9</v>
       </c>
       <c r="C35" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E35" t="s">
         <v>62</v>
@@ -1041,7 +1041,7 @@
         <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D40" t="s">
         <v>63</v>
@@ -1077,7 +1077,7 @@
         <v>7</v>
       </c>
       <c r="C44" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D44" t="s">
         <v>64</v>
@@ -1124,10 +1124,10 @@
         <v>37</v>
       </c>
       <c r="B49" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C49" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1146,7 +1146,7 @@
         <v>5</v>
       </c>
       <c r="C52" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D52" t="s">
         <v>65</v>
@@ -1237,7 +1237,7 @@
         <v>18</v>
       </c>
       <c r="C62" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E62" t="s">
         <v>45</v>
@@ -1298,7 +1298,7 @@
         <v>6</v>
       </c>
       <c r="C69" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D69" t="s">
         <v>73</v>
@@ -1375,10 +1375,10 @@
         <v>19</v>
       </c>
       <c r="B76" t="s">
+        <v>77</v>
+      </c>
+      <c r="C76" t="s">
         <v>78</v>
-      </c>
-      <c r="C76" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
@@ -1386,10 +1386,10 @@
         <v>19</v>
       </c>
       <c r="B77" t="s">
+        <v>79</v>
+      </c>
+      <c r="C77" t="s">
         <v>80</v>
-      </c>
-      <c r="C77" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -1408,7 +1408,7 @@
         <v>8</v>
       </c>
       <c r="C80" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D80" t="s">
         <v>66</v>

</xml_diff>

<commit_message>
Changed code1 (originall datEmpty.organizations.organizationID) to avoid circular references in ID generation
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B0AA56B-8624-9448-A1E4-922A9BA6E2B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB6EBA09-58FE-B949-8F8C-F30EA9ACC64C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
   <sheets>
     <sheet name="id_code" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="96">
   <si>
     <t>addresses</t>
   </si>
@@ -310,9 +310,6 @@
     <t>fn.makeid(dat.protocols.__protocolID)</t>
   </si>
   <si>
-    <t>datEmpty.organizations.organizationID</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures")))</t>
   </si>
   <si>
@@ -320,6 +317,12 @@
   </si>
   <si>
     <t>fn.makeid(datEmpty.protocolRelationships.protocolIDContainer, datEmpty.protocolRelationships.stepIDObj, datEmpty.protocolRelationships.relationshipID)</t>
+  </si>
+  <si>
+    <t>Having datEmpty.organizations.organizationID for code1 results in circular ID code.</t>
+  </si>
+  <si>
+    <t>fn.makeid("dataset")</t>
   </si>
 </sst>
 </file>
@@ -790,8 +793,11 @@
       <c r="C12" t="s">
         <v>85</v>
       </c>
-      <c r="D12" t="s">
-        <v>91</v>
+      <c r="D12" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -994,7 +1000,7 @@
         <v>9</v>
       </c>
       <c r="C35" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E35" t="s">
         <v>62</v>
@@ -1127,7 +1133,7 @@
         <v>76</v>
       </c>
       <c r="C49" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1237,7 +1243,7 @@
         <v>18</v>
       </c>
       <c r="C62" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E62" t="s">
         <v>45</v>

</xml_diff>

<commit_message>
Added sampleRelationships IDs and general updates
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB6EBA09-58FE-B949-8F8C-F30EA9ACC64C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148FFDD1-525D-394A-BDE9-CE6509A8AFBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
   <sheets>
     <sheet name="id_code" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="99">
   <si>
     <t>addresses</t>
   </si>
@@ -292,37 +292,46 @@
     <t>fn.makeid(dat.contacts.__contactID)</t>
   </si>
   <si>
+    <t>fn.makeid(dat.instruments.__instrumentID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.measures.__measureRepID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.organizations.__organizationID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.polygons.__polygonID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.protocols.__protocolID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures")))</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.qualityReports.qualityFlag, dat.qualityReports.measureRepID, dat.qualityReports.sampleID, dat.qualityReports.measureSetRepID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.protocolRelationships.protocolIDContainer, datEmpty.protocolRelationships.stepIDObj, datEmpty.protocolRelationships.relationshipID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.measures.__measureSetRepID)</t>
+  </si>
+  <si>
     <t>fn.makeid(dat.datasets.__datasetID)</t>
   </si>
   <si>
-    <t>fn.makeid(dat.instruments.__instrumentID)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.measures.__measureRepID)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.organizations.__organizationID)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.polygons.__polygonID)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.protocols.__protocolID)</t>
-  </si>
-  <si>
-    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures")))</t>
-  </si>
-  <si>
-    <t>fn.makeid(datEmpty.qualityReports.qualityFlag, dat.qualityReports.measureRepID, dat.qualityReports.sampleID, dat.qualityReports.measureSetRepID)</t>
-  </si>
-  <si>
-    <t>fn.makeid(datEmpty.protocolRelationships.protocolIDContainer, datEmpty.protocolRelationships.stepIDObj, datEmpty.protocolRelationships.relationshipID)</t>
-  </si>
-  <si>
-    <t>Having datEmpty.organizations.organizationID for code1 results in circular ID code.</t>
-  </si>
-  <si>
-    <t>fn.makeid("dataset")</t>
+    <t>fn.makeid(datEmpty.organizations.organizationID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.sampleRelationships.__sampleRelationshipsID)</t>
+  </si>
+  <si>
+    <t>fn.makeid("rel")</t>
+  </si>
+  <si>
+    <t>sampleRelationshipsID</t>
   </si>
 </sst>
 </file>
@@ -791,14 +800,12 @@
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>85</v>
-      </c>
-      <c r="D12" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D12" t="s">
         <v>95</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>94</v>
-      </c>
+      <c r="E12" s="1"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -840,7 +847,7 @@
         <v>16</v>
       </c>
       <c r="C18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D18" t="s">
         <v>60</v>
@@ -895,7 +902,7 @@
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D25" t="s">
         <v>61</v>
@@ -1000,7 +1007,10 @@
         <v>9</v>
       </c>
       <c r="C35" t="s">
-        <v>91</v>
+        <v>93</v>
+      </c>
+      <c r="D35" t="s">
+        <v>90</v>
       </c>
       <c r="E35" t="s">
         <v>62</v>
@@ -1047,7 +1057,7 @@
         <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D40" t="s">
         <v>63</v>
@@ -1083,7 +1093,7 @@
         <v>7</v>
       </c>
       <c r="C44" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D44" t="s">
         <v>64</v>
@@ -1133,7 +1143,7 @@
         <v>76</v>
       </c>
       <c r="C49" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1152,7 +1162,7 @@
         <v>5</v>
       </c>
       <c r="C52" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D52" t="s">
         <v>65</v>
@@ -1243,7 +1253,7 @@
         <v>18</v>
       </c>
       <c r="C62" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E62" t="s">
         <v>45</v>
@@ -1294,6 +1304,15 @@
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>38</v>
+      </c>
+      <c r="B67" t="s">
+        <v>98</v>
+      </c>
+      <c r="C67" t="s">
+        <v>96</v>
+      </c>
+      <c r="D67" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Add accessions table and other minor updates
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C49CD188-E612-5D43-B131-B38351535D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B9F757F-2EBB-EF4C-869C-D9BE0F9F9B85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="105">
   <si>
     <t>addresses</t>
   </si>
@@ -332,6 +332,24 @@
   </si>
   <si>
     <t>sampleRelationshipsID</t>
+  </si>
+  <si>
+    <t>accessions</t>
+  </si>
+  <si>
+    <t>accessIndexID</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.accessions.__accessIndexID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.accessions.organizationID, datEmpty.accessions.dataHost, datEmpty.accessions.accessNum)</t>
+  </si>
+  <si>
+    <t>fn.countrows("measures")</t>
+  </si>
+  <si>
+    <t>_extra_measures_count</t>
   </si>
 </sst>
 </file>
@@ -375,9 +393,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -692,7 +711,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A1991E-0020-B448-B50F-72C1AC9C88C8}">
-  <dimension ref="A1:E91"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -715,112 +734,115 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>46</v>
+    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D5" t="s">
-        <v>59</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="B6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>46</v>
+        <v>83</v>
+      </c>
+      <c r="D6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E6" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" t="s">
-        <v>2</v>
-      </c>
-      <c r="C12" t="s">
-        <v>94</v>
-      </c>
-      <c r="D12" t="s">
-        <v>95</v>
-      </c>
-      <c r="E12" s="1"/>
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -828,7 +850,7 @@
         <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -836,112 +858,101 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" t="s">
+        <v>95</v>
+      </c>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" t="s">
-        <v>85</v>
-      </c>
-      <c r="D18" t="s">
-        <v>60</v>
-      </c>
-      <c r="E18" t="s">
-        <v>68</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>2</v>
-      </c>
-      <c r="C19" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>32</v>
       </c>
-      <c r="B20" t="s">
-        <v>11</v>
-      </c>
-      <c r="C20" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>32</v>
-      </c>
-      <c r="B21" t="s">
-        <v>10</v>
-      </c>
-      <c r="C21" t="s">
-        <v>47</v>
+      <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" t="s">
+        <v>85</v>
+      </c>
+      <c r="D22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>33</v>
+        <v>32</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C23" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>86</v>
-      </c>
-      <c r="D25" t="s">
-        <v>61</v>
-      </c>
-      <c r="E25" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>3</v>
-      </c>
-      <c r="B26" t="s">
-        <v>5</v>
-      </c>
-      <c r="C26" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>3</v>
-      </c>
-      <c r="B27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C27" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B28" t="s">
-        <v>7</v>
-      </c>
-      <c r="C28" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -949,10 +960,16 @@
         <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>52</v>
+        <v>86</v>
+      </c>
+      <c r="D29" t="s">
+        <v>61</v>
+      </c>
+      <c r="E29" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -960,10 +977,10 @@
         <v>3</v>
       </c>
       <c r="B30" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -971,10 +988,10 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C31" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -982,10 +999,10 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C32" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -993,384 +1010,381 @@
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C33" t="s">
-        <v>48</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>3</v>
+      </c>
+      <c r="B34" t="s">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B35" t="s">
         <v>9</v>
       </c>
       <c r="C35" t="s">
-        <v>93</v>
-      </c>
-      <c r="D35" t="s">
-        <v>90</v>
-      </c>
-      <c r="E35" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C36" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B37" t="s">
+        <v>11</v>
+      </c>
+      <c r="C37" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
         <v>34</v>
       </c>
-      <c r="B37" t="s">
-        <v>10</v>
-      </c>
-      <c r="C37" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>34</v>
-      </c>
-      <c r="B38" t="s">
-        <v>11</v>
-      </c>
-      <c r="C38" t="s">
-        <v>48</v>
+      <c r="B39" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" t="s">
+        <v>93</v>
+      </c>
+      <c r="D39" t="s">
+        <v>90</v>
+      </c>
+      <c r="E39" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B40" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C40" t="s">
-        <v>87</v>
-      </c>
-      <c r="D40" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B41" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C42" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>36</v>
-      </c>
-      <c r="B44" t="s">
-        <v>7</v>
-      </c>
-      <c r="C44" t="s">
-        <v>88</v>
-      </c>
-      <c r="D44" t="s">
-        <v>64</v>
-      </c>
-      <c r="E44" t="s">
-        <v>64</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>34</v>
+      </c>
+      <c r="B43" t="s">
+        <v>104</v>
+      </c>
+      <c r="C43" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B45" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C45" t="s">
-        <v>46</v>
+        <v>87</v>
+      </c>
+      <c r="D45" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B46" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C46" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B47" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="C47" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B49" t="s">
-        <v>76</v>
+        <v>7</v>
       </c>
       <c r="C49" t="s">
-        <v>92</v>
+        <v>88</v>
+      </c>
+      <c r="D49" t="s">
+        <v>64</v>
+      </c>
+      <c r="E49" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>36</v>
+      </c>
+      <c r="B50" t="s">
+        <v>2</v>
+      </c>
+      <c r="C50" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="B51" t="s">
-        <v>13</v>
+        <v>10</v>
+      </c>
+      <c r="C51" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="B52" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C52" t="s">
-        <v>89</v>
-      </c>
-      <c r="D52" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>12</v>
-      </c>
-      <c r="B53" t="s">
-        <v>2</v>
-      </c>
-      <c r="C53" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
+        <v>37</v>
+      </c>
+      <c r="B54" t="s">
+        <v>76</v>
+      </c>
+      <c r="C54" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
         <v>12</v>
       </c>
-      <c r="B54" t="s">
-        <v>10</v>
-      </c>
-      <c r="C54" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>12</v>
-      </c>
-      <c r="B55" t="s">
-        <v>11</v>
-      </c>
-      <c r="C55" t="s">
-        <v>48</v>
+      <c r="B56" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C57" t="s">
-        <v>72</v>
+        <v>89</v>
+      </c>
+      <c r="D57" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C58" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B59" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C59" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B60" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C60" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B62" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C62" t="s">
-        <v>91</v>
-      </c>
-      <c r="E62" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B63" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C63" t="s">
-        <v>71</v>
-      </c>
-      <c r="E63" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B64" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C64" t="s">
-        <v>50</v>
-      </c>
-      <c r="E64" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B65" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C65" t="s">
-        <v>53</v>
-      </c>
-      <c r="E65" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="B67" t="s">
-        <v>98</v>
+        <v>18</v>
       </c>
       <c r="C67" t="s">
-        <v>96</v>
-      </c>
-      <c r="D67" t="s">
-        <v>97</v>
+        <v>91</v>
+      </c>
+      <c r="E67" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>17</v>
+      </c>
+      <c r="B68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C68" t="s">
+        <v>71</v>
+      </c>
+      <c r="E68" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B69" t="s">
         <v>6</v>
       </c>
       <c r="C69" t="s">
-        <v>82</v>
-      </c>
-      <c r="D69" t="s">
-        <v>73</v>
+        <v>50</v>
+      </c>
+      <c r="E69" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B70" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C70" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
-        <v>19</v>
-      </c>
-      <c r="B71" t="s">
-        <v>10</v>
-      </c>
-      <c r="C71" t="s">
-        <v>47</v>
+        <v>53</v>
+      </c>
+      <c r="E70" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B72" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="C72" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
-        <v>19</v>
-      </c>
-      <c r="B73" t="s">
-        <v>8</v>
-      </c>
-      <c r="C73" t="s">
-        <v>52</v>
+        <v>96</v>
+      </c>
+      <c r="D72" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
@@ -1378,10 +1392,13 @@
         <v>19</v>
       </c>
       <c r="B74" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C74" t="s">
-        <v>46</v>
+        <v>82</v>
+      </c>
+      <c r="D74" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.2">
@@ -1389,10 +1406,10 @@
         <v>19</v>
       </c>
       <c r="B75" t="s">
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="C75" t="s">
-        <v>75</v>
+        <v>49</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -1400,10 +1417,10 @@
         <v>19</v>
       </c>
       <c r="B76" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="C76" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
@@ -1411,112 +1428,167 @@
         <v>19</v>
       </c>
       <c r="B77" t="s">
-        <v>79</v>
+        <v>11</v>
       </c>
       <c r="C77" t="s">
-        <v>80</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>19</v>
+      </c>
+      <c r="B78" t="s">
+        <v>8</v>
+      </c>
+      <c r="C78" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B79" t="s">
-        <v>21</v>
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B80" t="s">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="C80" t="s">
-        <v>81</v>
-      </c>
-      <c r="D80" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B81" t="s">
-        <v>2</v>
+        <v>77</v>
       </c>
       <c r="C81" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B82" t="s">
-        <v>7</v>
+        <v>79</v>
       </c>
       <c r="C82" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>20</v>
-      </c>
-      <c r="B83" t="s">
-        <v>1</v>
-      </c>
-      <c r="C83" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>20</v>
       </c>
       <c r="B84" t="s">
-        <v>10</v>
-      </c>
-      <c r="C84" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>20</v>
       </c>
       <c r="B85" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C85" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+      <c r="D85" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>20</v>
       </c>
       <c r="B86" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>20</v>
       </c>
       <c r="B87" t="s">
+        <v>7</v>
+      </c>
+      <c r="C87" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>20</v>
+      </c>
+      <c r="B88" t="s">
+        <v>1</v>
+      </c>
+      <c r="C88" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>20</v>
+      </c>
+      <c r="B89" t="s">
+        <v>10</v>
+      </c>
+      <c r="C89" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>20</v>
+      </c>
+      <c r="B90" t="s">
+        <v>11</v>
+      </c>
+      <c r="C90" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>20</v>
+      </c>
+      <c r="B91" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>20</v>
+      </c>
+      <c r="B92" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
measureSets ID code changes
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B9F757F-2EBB-EF4C-869C-D9BE0F9F9B85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F61F3B7-9913-624B-AEBB-31372BD60B60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -307,18 +307,12 @@
     <t>fn.makeid(dat.protocols.__protocolID)</t>
   </si>
   <si>
-    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures")))</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.qualityReports.qualityFlag, dat.qualityReports.measureRepID, dat.qualityReports.sampleID, dat.qualityReports.measureSetRepID)</t>
   </si>
   <si>
     <t>fn.makeid(datEmpty.protocolRelationships.protocolIDContainer, datEmpty.protocolRelationships.stepIDObj, datEmpty.protocolRelationships.relationshipID)</t>
   </si>
   <si>
-    <t>fn.makeid(dat.measures.__measureSetRepID)</t>
-  </si>
-  <si>
     <t>fn.makeid(dat.datasets.__datasetID)</t>
   </si>
   <si>
@@ -350,6 +344,12 @@
   </si>
   <si>
     <t>_extra_measures_count</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.measures.__measureSetRepID) if int(dat.measureSets._extra_measures_count) else ""</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(int(dat.measureSets._extra_measures_count))) if int(dat.measureSets._extra_measures_count) else ""</t>
   </si>
 </sst>
 </file>
@@ -736,21 +736,21 @@
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>9</v>
@@ -761,7 +761,7 @@
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>10</v>
@@ -861,10 +861,10 @@
         <v>2</v>
       </c>
       <c r="C16" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E16" s="1"/>
     </row>
@@ -1068,10 +1068,10 @@
         <v>9</v>
       </c>
       <c r="C39" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="D39" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="E39" t="s">
         <v>62</v>
@@ -1115,10 +1115,10 @@
         <v>34</v>
       </c>
       <c r="B43" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C43" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -1215,7 +1215,7 @@
         <v>76</v>
       </c>
       <c r="C54" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
@@ -1325,7 +1325,7 @@
         <v>18</v>
       </c>
       <c r="C67" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E67" t="s">
         <v>45</v>
@@ -1378,13 +1378,13 @@
         <v>38</v>
       </c>
       <c r="B72" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C72" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D72" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Updates to accessions table
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F61F3B7-9913-624B-AEBB-31372BD60B60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB054B8E-E77B-F446-921F-DBFE40DDB15D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="105">
   <si>
     <t>addresses</t>
   </si>
@@ -393,10 +393,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -415,9 +414,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -455,7 +454,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -561,7 +560,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -703,7 +702,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -711,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A1991E-0020-B448-B50F-72C1AC9C88C8}">
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -734,74 +733,77 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>97</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
         <v>99</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>97</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C3" t="s">
         <v>47</v>
       </c>
     </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+    </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>0</v>
       </c>
       <c r="B6" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>83</v>
-      </c>
-      <c r="D6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E6" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C7" t="s">
         <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>84</v>
+      </c>
+      <c r="D8" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -809,13 +811,10 @@
         <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="C9" t="s">
-        <v>84</v>
-      </c>
-      <c r="D9" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -823,26 +822,23 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -850,30 +846,30 @@
         <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C15" t="s">
+        <v>92</v>
+      </c>
+      <c r="D15" t="s">
+        <v>93</v>
+      </c>
+      <c r="E15" s="1"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>2</v>
-      </c>
-      <c r="C16" t="s">
-        <v>92</v>
-      </c>
-      <c r="D16" t="s">
-        <v>93</v>
-      </c>
-      <c r="E16" s="1"/>
+        <v>28</v>
+      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -881,7 +877,7 @@
         <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -889,15 +885,24 @@
         <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>26</v>
-      </c>
-      <c r="B20" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" t="s">
+        <v>85</v>
+      </c>
+      <c r="D21" t="s">
+        <v>60</v>
+      </c>
+      <c r="E21" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -905,16 +910,10 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C22" t="s">
-        <v>85</v>
-      </c>
-      <c r="D22" t="s">
-        <v>60</v>
-      </c>
-      <c r="E22" t="s">
-        <v>68</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -922,10 +921,10 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
@@ -933,26 +932,32 @@
         <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>32</v>
-      </c>
-      <c r="B25" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" t="s">
+        <v>86</v>
+      </c>
+      <c r="D28" t="s">
+        <v>61</v>
+      </c>
+      <c r="E28" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -960,16 +965,10 @@
         <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>86</v>
-      </c>
-      <c r="D29" t="s">
-        <v>61</v>
-      </c>
-      <c r="E29" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -977,10 +976,10 @@
         <v>3</v>
       </c>
       <c r="B30" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C30" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -988,10 +987,10 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C31" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -999,10 +998,10 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C32" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -1010,10 +1009,10 @@
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C33" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
@@ -1021,10 +1020,10 @@
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C34" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
@@ -1032,10 +1031,10 @@
         <v>3</v>
       </c>
       <c r="B35" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C35" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1043,21 +1042,27 @@
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C36" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B37" t="s">
-        <v>11</v>
-      </c>
-      <c r="C37" t="s">
         <v>48</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" t="s">
+        <v>103</v>
+      </c>
+      <c r="D38" t="s">
+        <v>104</v>
+      </c>
+      <c r="E38" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -1065,16 +1070,10 @@
         <v>34</v>
       </c>
       <c r="B39" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C39" t="s">
-        <v>103</v>
-      </c>
-      <c r="D39" t="s">
-        <v>104</v>
-      </c>
-      <c r="E39" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
@@ -1082,10 +1081,10 @@
         <v>34</v>
       </c>
       <c r="B40" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -1093,10 +1092,10 @@
         <v>34</v>
       </c>
       <c r="B41" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C41" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -1104,21 +1103,24 @@
         <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>11</v>
+        <v>102</v>
       </c>
       <c r="C42" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>34</v>
-      </c>
-      <c r="B43" t="s">
-        <v>102</v>
-      </c>
-      <c r="C43" t="s">
         <v>101</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>35</v>
+      </c>
+      <c r="B44" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" t="s">
+        <v>87</v>
+      </c>
+      <c r="D44" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -1126,13 +1128,10 @@
         <v>35</v>
       </c>
       <c r="B45" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>87</v>
-      </c>
-      <c r="D45" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
@@ -1140,181 +1139,184 @@
         <v>35</v>
       </c>
       <c r="B46" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C46" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>35</v>
-      </c>
-      <c r="B47" t="s">
-        <v>2</v>
-      </c>
-      <c r="C47" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>36</v>
+      </c>
+      <c r="B48" t="s">
+        <v>7</v>
+      </c>
+      <c r="C48" t="s">
+        <v>88</v>
+      </c>
+      <c r="D48" t="s">
+        <v>64</v>
+      </c>
+      <c r="E48" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>36</v>
       </c>
       <c r="B49" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C49" t="s">
-        <v>88</v>
-      </c>
-      <c r="D49" t="s">
-        <v>64</v>
-      </c>
-      <c r="E49" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>36</v>
       </c>
       <c r="B50" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C50" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>36</v>
       </c>
       <c r="B51" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C51" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>36</v>
-      </c>
-      <c r="B52" t="s">
-        <v>11</v>
-      </c>
-      <c r="C52" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
         <v>37</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B53" t="s">
         <v>76</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C53" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>12</v>
+      </c>
+      <c r="B55" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>12</v>
       </c>
       <c r="B56" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="C56" t="s">
+        <v>89</v>
+      </c>
+      <c r="D56" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C57" t="s">
-        <v>89</v>
-      </c>
-      <c r="D57" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C58" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>12</v>
       </c>
       <c r="B59" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C59" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>12</v>
-      </c>
-      <c r="B60" t="s">
-        <v>11</v>
-      </c>
-      <c r="C60" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>14</v>
+      </c>
+      <c r="B61" t="s">
+        <v>15</v>
+      </c>
+      <c r="C61" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>14</v>
       </c>
       <c r="B62" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C62" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>14</v>
       </c>
       <c r="B63" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C63" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>14</v>
       </c>
       <c r="B64" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C64" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>14</v>
-      </c>
-      <c r="B65" t="s">
-        <v>16</v>
-      </c>
-      <c r="C65" t="s">
         <v>55</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>17</v>
+      </c>
+      <c r="B66" t="s">
+        <v>18</v>
+      </c>
+      <c r="C66" t="s">
+        <v>90</v>
+      </c>
+      <c r="E66" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
@@ -1322,13 +1324,13 @@
         <v>17</v>
       </c>
       <c r="B67" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C67" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="E67" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
@@ -1336,13 +1338,13 @@
         <v>17</v>
       </c>
       <c r="B68" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C68" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="E68" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
@@ -1350,41 +1352,41 @@
         <v>17</v>
       </c>
       <c r="B69" t="s">
+        <v>9</v>
+      </c>
+      <c r="C69" t="s">
+        <v>53</v>
+      </c>
+      <c r="E69" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>38</v>
+      </c>
+      <c r="B71" t="s">
+        <v>96</v>
+      </c>
+      <c r="C71" t="s">
+        <v>94</v>
+      </c>
+      <c r="D71" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>19</v>
+      </c>
+      <c r="B73" t="s">
         <v>6</v>
       </c>
-      <c r="C69" t="s">
-        <v>50</v>
-      </c>
-      <c r="E69" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
-        <v>17</v>
-      </c>
-      <c r="B70" t="s">
-        <v>9</v>
-      </c>
-      <c r="C70" t="s">
-        <v>53</v>
-      </c>
-      <c r="E70" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
-        <v>38</v>
-      </c>
-      <c r="B72" t="s">
-        <v>96</v>
-      </c>
-      <c r="C72" t="s">
-        <v>94</v>
-      </c>
-      <c r="D72" t="s">
-        <v>95</v>
+      <c r="C73" t="s">
+        <v>82</v>
+      </c>
+      <c r="D73" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
@@ -1392,13 +1394,10 @@
         <v>19</v>
       </c>
       <c r="B74" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C74" t="s">
-        <v>82</v>
-      </c>
-      <c r="D74" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.2">
@@ -1406,10 +1405,10 @@
         <v>19</v>
       </c>
       <c r="B75" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C75" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -1417,10 +1416,10 @@
         <v>19</v>
       </c>
       <c r="B76" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C76" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
@@ -1428,10 +1427,10 @@
         <v>19</v>
       </c>
       <c r="B77" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C77" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
@@ -1439,10 +1438,10 @@
         <v>19</v>
       </c>
       <c r="B78" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C78" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -1450,10 +1449,10 @@
         <v>19</v>
       </c>
       <c r="B79" t="s">
-        <v>2</v>
+        <v>70</v>
       </c>
       <c r="C79" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
@@ -1461,10 +1460,10 @@
         <v>19</v>
       </c>
       <c r="B80" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C80" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
@@ -1472,21 +1471,18 @@
         <v>19</v>
       </c>
       <c r="B81" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C81" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>19</v>
-      </c>
-      <c r="B82" t="s">
-        <v>79</v>
-      </c>
-      <c r="C82" t="s">
         <v>80</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>20</v>
+      </c>
+      <c r="B83" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
@@ -1494,7 +1490,13 @@
         <v>20</v>
       </c>
       <c r="B84" t="s">
-        <v>21</v>
+        <v>8</v>
+      </c>
+      <c r="C84" t="s">
+        <v>81</v>
+      </c>
+      <c r="D84" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
@@ -1502,13 +1504,10 @@
         <v>20</v>
       </c>
       <c r="B85" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C85" t="s">
-        <v>81</v>
-      </c>
-      <c r="D85" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
@@ -1516,10 +1515,10 @@
         <v>20</v>
       </c>
       <c r="B86" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C86" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
@@ -1527,10 +1526,10 @@
         <v>20</v>
       </c>
       <c r="B87" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C87" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
@@ -1538,10 +1537,10 @@
         <v>20</v>
       </c>
       <c r="B88" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C88" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
@@ -1549,10 +1548,10 @@
         <v>20</v>
       </c>
       <c r="B89" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C89" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
@@ -1560,10 +1559,7 @@
         <v>20</v>
       </c>
       <c r="B90" t="s">
-        <v>11</v>
-      </c>
-      <c r="C90" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
@@ -1571,24 +1567,16 @@
         <v>20</v>
       </c>
       <c r="B91" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
-        <v>20</v>
-      </c>
-      <c r="B92" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updates to general ODM v2 ID code. Set some primary keys to blank when data is missing.
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB054B8E-E77B-F446-921F-DBFE40DDB15D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D134200D-F0C1-6246-A21D-FA4F7719528C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="111">
   <si>
     <t>addresses</t>
   </si>
@@ -214,9 +214,6 @@
     <t>dat.measureSets.measureSetRepID if dat.qualityReports.__measureSetRepID else ""</t>
   </si>
   <si>
-    <t>fn.makeid(datEmpty.organizations.organizationID, datEmpty.contacts.role[:3])</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.instruments.manufacturer, datEmpty.instruments.name[:3], datEmpty.instruments.model[:3])</t>
   </si>
   <si>
@@ -232,9 +229,6 @@
     <t>fn.makeid(datEmpty.organizations.organizationID, datEmpty.sites.siteID)</t>
   </si>
   <si>
-    <t>fn.makeid(datEmpty.protocols.name, datEmpty.protocols.protocolVersion)</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.addresses.country, datEmpty.addresses.pCode, datEmpty.addresses.city[:3], datEmpty.sites.name[:3])</t>
   </si>
   <si>
@@ -289,9 +283,6 @@
     <t>fn.makeid(dat.addresses.__addressID)</t>
   </si>
   <si>
-    <t>fn.makeid(dat.contacts.__contactID)</t>
-  </si>
-  <si>
     <t>fn.makeid(dat.instruments.__instrumentID)</t>
   </si>
   <si>
@@ -304,9 +295,6 @@
     <t>fn.makeid(dat.polygons.__polygonID)</t>
   </si>
   <si>
-    <t>fn.makeid(dat.protocols.__protocolID)</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.qualityReports.qualityFlag, dat.qualityReports.measureRepID, dat.qualityReports.sampleID, dat.qualityReports.measureSetRepID)</t>
   </si>
   <si>
@@ -350,6 +338,36 @@
   </si>
   <si>
     <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(int(dat.measureSets._extra_measures_count))) if int(dat.measureSets._extra_measures_count) else ""</t>
+  </si>
+  <si>
+    <t>_extra_protocolSteps_count</t>
+  </si>
+  <si>
+    <t>fn.countrows("protocolSteps")</t>
+  </si>
+  <si>
+    <t>_extra_fk_count</t>
+  </si>
+  <si>
+    <t>int(dat.protocols._extra_measures_count) + int(dat.protocols._extra_protocolSteps_count)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.protocols.__protocolID) if int(dat.protocols._extra_fk_count) else ""</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.protocols.name, datEmpty.protocols.protocolVersion) if int(dat.protocols._extra_fk_count) else ""</t>
+  </si>
+  <si>
+    <t>_extra_has_data</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.contacts.__contactID) if dat.contacts._extra_has_data else ""</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.organizations.organizationID, datEmpty.contacts.role[:3]) if dat.contacts._extra_has_data else ""</t>
+  </si>
+  <si>
+    <t>True if (dat.contacts.firstName or dat.contacts.lastName or dat.contacts.email or dat.contacts.coPhone or dat.contacts.role) else ""</t>
   </si>
 </sst>
 </file>
@@ -710,12 +728,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A1991E-0020-B448-B50F-72C1AC9C88C8}">
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="81.6640625" customWidth="1"/>
+    <col min="3" max="3" width="136.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="113" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -735,21 +753,21 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
@@ -772,13 +790,13 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -800,10 +818,10 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="D8" t="s">
-        <v>59</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -828,17 +846,20 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -846,30 +867,30 @@
         <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>2</v>
-      </c>
-      <c r="C15" t="s">
-        <v>92</v>
-      </c>
-      <c r="D15" t="s">
-        <v>93</v>
-      </c>
-      <c r="E15" s="1"/>
+        <v>27</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" t="s">
+        <v>89</v>
+      </c>
+      <c r="E16" s="1"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -877,7 +898,7 @@
         <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -885,24 +906,15 @@
         <v>26</v>
       </c>
       <c r="B19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>32</v>
-      </c>
-      <c r="B21" t="s">
-        <v>16</v>
-      </c>
-      <c r="C21" t="s">
-        <v>85</v>
-      </c>
-      <c r="D21" t="s">
-        <v>60</v>
-      </c>
-      <c r="E21" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -910,10 +922,16 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C22" t="s">
-        <v>46</v>
+        <v>82</v>
+      </c>
+      <c r="D22" t="s">
+        <v>59</v>
+      </c>
+      <c r="E22" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -921,10 +939,10 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="C23" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
@@ -932,32 +950,26 @@
         <v>32</v>
       </c>
       <c r="B24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" t="s">
         <v>10</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C25" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B28" t="s">
-        <v>4</v>
-      </c>
-      <c r="C28" t="s">
-        <v>86</v>
-      </c>
-      <c r="D28" t="s">
-        <v>61</v>
-      </c>
-      <c r="E28" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -965,10 +977,16 @@
         <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>49</v>
+        <v>83</v>
+      </c>
+      <c r="D29" t="s">
+        <v>60</v>
+      </c>
+      <c r="E29" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -976,10 +994,10 @@
         <v>3</v>
       </c>
       <c r="B30" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -987,10 +1005,10 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C31" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -998,10 +1016,10 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C32" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -1009,10 +1027,10 @@
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C33" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
@@ -1020,10 +1038,10 @@
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C34" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
@@ -1031,10 +1049,10 @@
         <v>3</v>
       </c>
       <c r="B35" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C35" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1042,27 +1060,21 @@
         <v>3</v>
       </c>
       <c r="B36" t="s">
+        <v>10</v>
+      </c>
+      <c r="C36" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B37" t="s">
         <v>11</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C37" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>34</v>
-      </c>
-      <c r="B38" t="s">
-        <v>9</v>
-      </c>
-      <c r="C38" t="s">
-        <v>103</v>
-      </c>
-      <c r="D38" t="s">
-        <v>104</v>
-      </c>
-      <c r="E38" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -1070,10 +1082,16 @@
         <v>34</v>
       </c>
       <c r="B39" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C39" t="s">
-        <v>49</v>
+        <v>99</v>
+      </c>
+      <c r="D39" t="s">
+        <v>100</v>
+      </c>
+      <c r="E39" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
@@ -1081,10 +1099,10 @@
         <v>34</v>
       </c>
       <c r="B40" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C40" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -1092,10 +1110,10 @@
         <v>34</v>
       </c>
       <c r="B41" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -1103,24 +1121,21 @@
         <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="C42" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>35</v>
-      </c>
-      <c r="B44" t="s">
-        <v>10</v>
-      </c>
-      <c r="C44" t="s">
-        <v>87</v>
-      </c>
-      <c r="D44" t="s">
-        <v>63</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>34</v>
+      </c>
+      <c r="B43" t="s">
+        <v>98</v>
+      </c>
+      <c r="C43" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -1128,10 +1143,13 @@
         <v>35</v>
       </c>
       <c r="B45" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C45" t="s">
-        <v>54</v>
+        <v>84</v>
+      </c>
+      <c r="D45" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
@@ -1139,298 +1157,284 @@
         <v>35</v>
       </c>
       <c r="B46" t="s">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>35</v>
+      </c>
+      <c r="B47" t="s">
         <v>2</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C47" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>36</v>
-      </c>
-      <c r="B48" t="s">
-        <v>7</v>
-      </c>
-      <c r="C48" t="s">
-        <v>88</v>
-      </c>
-      <c r="D48" t="s">
-        <v>64</v>
-      </c>
-      <c r="E48" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>36</v>
       </c>
       <c r="B49" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C49" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+      <c r="D49" t="s">
+        <v>63</v>
+      </c>
+      <c r="E49" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>36</v>
       </c>
       <c r="B50" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C50" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>36</v>
       </c>
       <c r="B51" t="s">
+        <v>10</v>
+      </c>
+      <c r="C51" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>36</v>
+      </c>
+      <c r="B52" t="s">
         <v>11</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C52" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
         <v>37</v>
       </c>
-      <c r="B53" t="s">
-        <v>76</v>
-      </c>
-      <c r="C53" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>12</v>
-      </c>
-      <c r="B55" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B54" t="s">
+        <v>74</v>
+      </c>
+      <c r="C54" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>12</v>
       </c>
       <c r="B56" t="s">
-        <v>5</v>
-      </c>
-      <c r="C56" t="s">
-        <v>89</v>
-      </c>
-      <c r="D56" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C57" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+      <c r="D57" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C58" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>12</v>
       </c>
       <c r="B59" t="s">
+        <v>10</v>
+      </c>
+      <c r="C59" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>12</v>
+      </c>
+      <c r="B60" t="s">
         <v>11</v>
       </c>
-      <c r="C59" t="s">
+      <c r="C60" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B61" t="s">
-        <v>15</v>
+        <v>98</v>
       </c>
       <c r="C61" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B62" t="s">
-        <v>10</v>
+        <v>101</v>
       </c>
       <c r="C62" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B63" t="s">
-        <v>11</v>
+        <v>103</v>
       </c>
       <c r="C63" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
-        <v>14</v>
-      </c>
-      <c r="B64" t="s">
-        <v>16</v>
-      </c>
-      <c r="C64" t="s">
-        <v>55</v>
+        <v>104</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B66" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C66" t="s">
-        <v>90</v>
-      </c>
-      <c r="E66" t="s">
-        <v>45</v>
+        <v>70</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B67" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C67" t="s">
-        <v>71</v>
-      </c>
-      <c r="E67" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B68" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C68" t="s">
-        <v>50</v>
-      </c>
-      <c r="E68" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B69" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C69" t="s">
-        <v>53</v>
-      </c>
-      <c r="E69" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="B71" t="s">
-        <v>96</v>
+        <v>18</v>
       </c>
       <c r="C71" t="s">
-        <v>94</v>
-      </c>
-      <c r="D71" t="s">
-        <v>95</v>
+        <v>86</v>
+      </c>
+      <c r="E71" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>17</v>
+      </c>
+      <c r="B72" t="s">
+        <v>4</v>
+      </c>
+      <c r="C72" t="s">
+        <v>69</v>
+      </c>
+      <c r="E72" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B73" t="s">
         <v>6</v>
       </c>
       <c r="C73" t="s">
-        <v>82</v>
-      </c>
-      <c r="D73" t="s">
-        <v>73</v>
+        <v>50</v>
+      </c>
+      <c r="E73" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B74" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C74" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
-        <v>19</v>
-      </c>
-      <c r="B75" t="s">
-        <v>10</v>
-      </c>
-      <c r="C75" t="s">
-        <v>47</v>
+        <v>53</v>
+      </c>
+      <c r="E74" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B76" t="s">
-        <v>11</v>
+        <v>92</v>
       </c>
       <c r="C76" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
-        <v>19</v>
-      </c>
-      <c r="B77" t="s">
-        <v>8</v>
-      </c>
-      <c r="C77" t="s">
-        <v>52</v>
+        <v>90</v>
+      </c>
+      <c r="D76" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
@@ -1438,10 +1442,13 @@
         <v>19</v>
       </c>
       <c r="B78" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C78" t="s">
-        <v>46</v>
+        <v>80</v>
+      </c>
+      <c r="D78" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -1449,10 +1456,7 @@
         <v>19</v>
       </c>
       <c r="B79" t="s">
-        <v>70</v>
-      </c>
-      <c r="C79" t="s">
-        <v>75</v>
+        <v>5</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
@@ -1460,10 +1464,10 @@
         <v>19</v>
       </c>
       <c r="B80" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="C80" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
@@ -1471,65 +1475,65 @@
         <v>19</v>
       </c>
       <c r="B81" t="s">
-        <v>79</v>
+        <v>11</v>
       </c>
       <c r="C81" t="s">
-        <v>80</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>19</v>
+      </c>
+      <c r="B82" t="s">
+        <v>8</v>
+      </c>
+      <c r="C82" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B83" t="s">
-        <v>21</v>
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B84" t="s">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="C84" t="s">
-        <v>81</v>
-      </c>
-      <c r="D84" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B85" t="s">
-        <v>2</v>
+        <v>75</v>
       </c>
       <c r="C85" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B86" t="s">
-        <v>7</v>
+        <v>77</v>
       </c>
       <c r="C86" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
-        <v>20</v>
-      </c>
-      <c r="B87" t="s">
-        <v>1</v>
-      </c>
-      <c r="C87" t="s">
-        <v>54</v>
+        <v>78</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
@@ -1537,10 +1541,7 @@
         <v>20</v>
       </c>
       <c r="B88" t="s">
-        <v>10</v>
-      </c>
-      <c r="C88" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
@@ -1548,10 +1549,13 @@
         <v>20</v>
       </c>
       <c r="B89" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C89" t="s">
-        <v>48</v>
+        <v>79</v>
+      </c>
+      <c r="D89" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
@@ -1559,7 +1563,10 @@
         <v>20</v>
       </c>
       <c r="B90" t="s">
-        <v>22</v>
+        <v>2</v>
+      </c>
+      <c r="C90" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
@@ -1567,16 +1574,68 @@
         <v>20</v>
       </c>
       <c r="B91" t="s">
-        <v>23</v>
+        <v>7</v>
+      </c>
+      <c r="C91" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>20</v>
+      </c>
+      <c r="B92" t="s">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>39</v>
+        <v>20</v>
+      </c>
+      <c r="B93" t="s">
+        <v>10</v>
+      </c>
+      <c r="C93" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>20</v>
+      </c>
+      <c r="B94" t="s">
+        <v>11</v>
+      </c>
+      <c r="C94" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
+        <v>20</v>
+      </c>
+      <c r="B95" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>20</v>
+      </c>
+      <c r="B96" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
General updates to ODM v2 code
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D134200D-F0C1-6246-A21D-FA4F7719528C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05278200-CEEA-3346-B3B9-6A74A8816150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="111">
   <si>
     <t>addresses</t>
   </si>
@@ -728,7 +728,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A1991E-0020-B448-B50F-72C1AC9C88C8}">
-  <dimension ref="A1:E100"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -939,37 +939,43 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C23" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>32</v>
-      </c>
-      <c r="B24" t="s">
-        <v>11</v>
-      </c>
-      <c r="C24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>32</v>
-      </c>
-      <c r="B25" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>33</v>
+        <v>3</v>
+      </c>
+      <c r="B27" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" t="s">
+        <v>83</v>
+      </c>
+      <c r="D27" t="s">
+        <v>60</v>
+      </c>
+      <c r="E27" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" t="s">
+        <v>5</v>
+      </c>
+      <c r="C28" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -977,16 +983,10 @@
         <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C29" t="s">
-        <v>83</v>
-      </c>
-      <c r="D29" t="s">
-        <v>60</v>
-      </c>
-      <c r="E29" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -994,10 +994,10 @@
         <v>3</v>
       </c>
       <c r="B30" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C30" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1005,10 +1005,10 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C31" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -1016,10 +1016,10 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C32" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -1027,10 +1027,10 @@
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C33" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
@@ -1038,10 +1038,10 @@
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
@@ -1049,32 +1049,38 @@
         <v>3</v>
       </c>
       <c r="B35" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C35" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>3</v>
-      </c>
-      <c r="B36" t="s">
-        <v>10</v>
-      </c>
-      <c r="C36" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="B37" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C37" t="s">
-        <v>48</v>
+        <v>99</v>
+      </c>
+      <c r="D37" t="s">
+        <v>100</v>
+      </c>
+      <c r="E37" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" t="s">
+        <v>5</v>
+      </c>
+      <c r="C38" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -1082,16 +1088,10 @@
         <v>34</v>
       </c>
       <c r="B39" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>99</v>
-      </c>
-      <c r="D39" t="s">
-        <v>100</v>
-      </c>
-      <c r="E39" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
@@ -1099,10 +1099,10 @@
         <v>34</v>
       </c>
       <c r="B40" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C40" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -1110,62 +1110,57 @@
         <v>34</v>
       </c>
       <c r="B41" t="s">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="C41" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>34</v>
-      </c>
-      <c r="B42" t="s">
-        <v>11</v>
-      </c>
-      <c r="C42" t="s">
-        <v>48</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="C43" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+        <v>84</v>
+      </c>
+      <c r="D43" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
         <v>35</v>
       </c>
-      <c r="B45" t="s">
-        <v>10</v>
-      </c>
-      <c r="C45" t="s">
-        <v>84</v>
-      </c>
-      <c r="D45" t="s">
-        <v>62</v>
+      <c r="B44" t="s">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B46" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C46" t="s">
-        <v>54</v>
+        <v>85</v>
+      </c>
+      <c r="D46" t="s">
+        <v>63</v>
+      </c>
+      <c r="E46" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B47" t="s">
         <v>2</v>
@@ -1174,153 +1169,158 @@
         <v>46</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>36</v>
+      </c>
+      <c r="B48" t="s">
+        <v>10</v>
+      </c>
+      <c r="C48" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>36</v>
       </c>
       <c r="B49" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C49" t="s">
-        <v>85</v>
-      </c>
-      <c r="D49" t="s">
-        <v>63</v>
-      </c>
-      <c r="E49" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B50" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>37</v>
+      </c>
+      <c r="B51" t="s">
+        <v>74</v>
+      </c>
+      <c r="C51" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>12</v>
+      </c>
+      <c r="B53" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>12</v>
+      </c>
+      <c r="B54" t="s">
+        <v>5</v>
+      </c>
+      <c r="C54" t="s">
+        <v>105</v>
+      </c>
+      <c r="D54" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>12</v>
+      </c>
+      <c r="B55" t="s">
         <v>2</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C55" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>36</v>
-      </c>
-      <c r="B51" t="s">
-        <v>10</v>
-      </c>
-      <c r="C51" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>36</v>
-      </c>
-      <c r="B52" t="s">
-        <v>11</v>
-      </c>
-      <c r="C52" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>37</v>
-      </c>
-      <c r="B54" t="s">
-        <v>74</v>
-      </c>
-      <c r="C54" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>12</v>
       </c>
       <c r="B56" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="C56" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C57" t="s">
-        <v>105</v>
-      </c>
-      <c r="D57" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>2</v>
+        <v>98</v>
       </c>
       <c r="C58" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>12</v>
       </c>
       <c r="B59" t="s">
-        <v>10</v>
+        <v>101</v>
       </c>
       <c r="C59" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>12</v>
       </c>
       <c r="B60" t="s">
+        <v>103</v>
+      </c>
+      <c r="C60" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>14</v>
+      </c>
+      <c r="B63" t="s">
+        <v>15</v>
+      </c>
+      <c r="C63" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>14</v>
+      </c>
+      <c r="B64" t="s">
+        <v>10</v>
+      </c>
+      <c r="C64" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>14</v>
+      </c>
+      <c r="B65" t="s">
         <v>11</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C65" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
-        <v>12</v>
-      </c>
-      <c r="B61" t="s">
-        <v>98</v>
-      </c>
-      <c r="C61" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>12</v>
-      </c>
-      <c r="B62" t="s">
-        <v>101</v>
-      </c>
-      <c r="C62" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>12</v>
-      </c>
-      <c r="B63" t="s">
-        <v>103</v>
-      </c>
-      <c r="C63" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
@@ -1328,43 +1328,52 @@
         <v>14</v>
       </c>
       <c r="B66" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C66" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
-        <v>14</v>
-      </c>
-      <c r="B67" t="s">
-        <v>10</v>
-      </c>
-      <c r="C67" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B68" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C68" t="s">
-        <v>48</v>
+        <v>86</v>
+      </c>
+      <c r="E68" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B69" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C69" t="s">
-        <v>55</v>
+        <v>69</v>
+      </c>
+      <c r="E69" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>17</v>
+      </c>
+      <c r="B70" t="s">
+        <v>6</v>
+      </c>
+      <c r="C70" t="s">
+        <v>50</v>
+      </c>
+      <c r="E70" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.2">
@@ -1372,69 +1381,60 @@
         <v>17</v>
       </c>
       <c r="B71" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="C71" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="E71" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
-        <v>17</v>
-      </c>
-      <c r="B72" t="s">
-        <v>4</v>
-      </c>
-      <c r="C72" t="s">
-        <v>69</v>
-      </c>
-      <c r="E72" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="B73" t="s">
+        <v>92</v>
+      </c>
+      <c r="C73" t="s">
+        <v>90</v>
+      </c>
+      <c r="D73" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>19</v>
+      </c>
+      <c r="B75" t="s">
         <v>6</v>
       </c>
-      <c r="C73" t="s">
-        <v>50</v>
-      </c>
-      <c r="E73" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
-        <v>17</v>
-      </c>
-      <c r="B74" t="s">
-        <v>9</v>
-      </c>
-      <c r="C74" t="s">
-        <v>53</v>
-      </c>
-      <c r="E74" t="s">
-        <v>58</v>
+      <c r="C75" t="s">
+        <v>80</v>
+      </c>
+      <c r="D75" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="B76" t="s">
-        <v>92</v>
-      </c>
-      <c r="C76" t="s">
-        <v>90</v>
-      </c>
-      <c r="D76" t="s">
-        <v>91</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>19</v>
+      </c>
+      <c r="B77" t="s">
+        <v>10</v>
+      </c>
+      <c r="C77" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
@@ -1442,13 +1442,10 @@
         <v>19</v>
       </c>
       <c r="B78" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C78" t="s">
-        <v>80</v>
-      </c>
-      <c r="D78" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -1456,7 +1453,10 @@
         <v>19</v>
       </c>
       <c r="B79" t="s">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="C79" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
@@ -1464,10 +1464,10 @@
         <v>19</v>
       </c>
       <c r="B80" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C80" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
@@ -1475,10 +1475,10 @@
         <v>19</v>
       </c>
       <c r="B81" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="C81" t="s">
-        <v>48</v>
+        <v>73</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
@@ -1486,10 +1486,10 @@
         <v>19</v>
       </c>
       <c r="B82" t="s">
-        <v>8</v>
+        <v>75</v>
       </c>
       <c r="C82" t="s">
-        <v>52</v>
+        <v>76</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
@@ -1497,43 +1497,43 @@
         <v>19</v>
       </c>
       <c r="B83" t="s">
-        <v>2</v>
+        <v>77</v>
       </c>
       <c r="C83" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
-        <v>19</v>
-      </c>
-      <c r="B84" t="s">
-        <v>68</v>
-      </c>
-      <c r="C84" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B85" t="s">
-        <v>75</v>
-      </c>
-      <c r="C85" t="s">
-        <v>76</v>
+        <v>21</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B86" t="s">
-        <v>77</v>
+        <v>8</v>
       </c>
       <c r="C86" t="s">
-        <v>78</v>
+        <v>79</v>
+      </c>
+      <c r="D86" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>20</v>
+      </c>
+      <c r="B87" t="s">
+        <v>2</v>
+      </c>
+      <c r="C87" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
@@ -1541,7 +1541,10 @@
         <v>20</v>
       </c>
       <c r="B88" t="s">
-        <v>21</v>
+        <v>7</v>
+      </c>
+      <c r="C88" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
@@ -1549,13 +1552,10 @@
         <v>20</v>
       </c>
       <c r="B89" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C89" t="s">
-        <v>79</v>
-      </c>
-      <c r="D89" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
@@ -1563,10 +1563,10 @@
         <v>20</v>
       </c>
       <c r="B90" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C90" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
@@ -1574,10 +1574,10 @@
         <v>20</v>
       </c>
       <c r="B91" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C91" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
@@ -1585,10 +1585,7 @@
         <v>20</v>
       </c>
       <c r="B92" t="s">
-        <v>1</v>
-      </c>
-      <c r="C92" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
@@ -1596,46 +1593,16 @@
         <v>20</v>
       </c>
       <c r="B93" t="s">
-        <v>10</v>
-      </c>
-      <c r="C93" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
-        <v>20</v>
-      </c>
-      <c r="B94" t="s">
-        <v>11</v>
-      </c>
-      <c r="C94" t="s">
-        <v>48</v>
+        <v>23</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>20</v>
-      </c>
-      <c r="B95" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
-        <v>20</v>
-      </c>
-      <c r="B96" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
General updates to ID generation code
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05278200-CEEA-3346-B3B9-6A74A8816150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{854DE97F-5196-A44F-B2B6-C29DF46C9CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="113">
   <si>
     <t>addresses</t>
   </si>
@@ -244,9 +244,6 @@
     <t>collDT</t>
   </si>
   <si>
-    <t>dat.measures.measureRepID</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.organizations.organizationID, datEmpty.protocolSteps.measure[-3:] if dat.protocolSteps.measure else datEmpty.protocolSteps.method[-3:])</t>
   </si>
   <si>
@@ -368,6 +365,15 @@
   </si>
   <si>
     <t>True if (dat.contacts.firstName or dat.contacts.lastName or dat.contacts.email or dat.contacts.coPhone or dat.contacts.role) else ""</t>
+  </si>
+  <si>
+    <t>dat.contacts.get_first_linked_value("contactID", linkage_path="datasets_to_contacts_funderCont_contactID")</t>
+  </si>
+  <si>
+    <t>dat.contacts.get_first_linked_value("contactID", linkage_path="datasets_to_contacts_custodyCont_contactID")</t>
+  </si>
+  <si>
+    <t>dat.measures.get_first_linked_value("measureRepID", linkage_path="qualityReports_to_measures_measure")</t>
   </si>
 </sst>
 </file>
@@ -728,7 +734,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A1991E-0020-B448-B50F-72C1AC9C88C8}">
-  <dimension ref="A1:E97"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -753,21 +759,21 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" t="s">
         <v>93</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>94</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>95</v>
-      </c>
-      <c r="D2" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
@@ -790,10 +796,10 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E5" t="s">
         <v>65</v>
@@ -818,10 +824,10 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D8" t="s">
         <v>108</v>
-      </c>
-      <c r="D8" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -829,10 +835,10 @@
         <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -840,26 +846,23 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>106</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" t="s">
-        <v>107</v>
-      </c>
-      <c r="C11" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -867,30 +870,36 @@
         <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C15" t="s">
+        <v>87</v>
+      </c>
+      <c r="D15" t="s">
+        <v>88</v>
+      </c>
+      <c r="E15" s="1"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
-      </c>
-      <c r="D16" t="s">
-        <v>89</v>
-      </c>
-      <c r="E16" s="1"/>
+        <v>110</v>
+      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="C17" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -898,7 +907,7 @@
         <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -906,15 +915,27 @@
         <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>26</v>
-      </c>
-      <c r="B20" t="s">
         <v>31</v>
+      </c>
+      <c r="C19" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" t="s">
+        <v>59</v>
+      </c>
+      <c r="E21" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -922,32 +943,32 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C22" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
         <v>82</v>
       </c>
-      <c r="D22" t="s">
-        <v>59</v>
-      </c>
-      <c r="E22" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>32</v>
-      </c>
-      <c r="B23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C23" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>33</v>
+      <c r="D26" t="s">
+        <v>60</v>
+      </c>
+      <c r="E26" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -955,16 +976,10 @@
         <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C27" t="s">
-        <v>83</v>
-      </c>
-      <c r="D27" t="s">
-        <v>60</v>
-      </c>
-      <c r="E27" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -972,10 +987,10 @@
         <v>3</v>
       </c>
       <c r="B28" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C28" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -983,10 +998,10 @@
         <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C29" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -994,10 +1009,10 @@
         <v>3</v>
       </c>
       <c r="B30" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C30" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1005,10 +1020,10 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C31" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -1016,10 +1031,10 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C32" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -1027,10 +1042,10 @@
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
@@ -1038,21 +1053,27 @@
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C34" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>3</v>
-      </c>
-      <c r="B35" t="s">
-        <v>11</v>
-      </c>
-      <c r="C35" t="s">
         <v>48</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>34</v>
+      </c>
+      <c r="B36" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" t="s">
+        <v>98</v>
+      </c>
+      <c r="D36" t="s">
+        <v>99</v>
+      </c>
+      <c r="E36" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1060,16 +1081,10 @@
         <v>34</v>
       </c>
       <c r="B37" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C37" t="s">
-        <v>99</v>
-      </c>
-      <c r="D37" t="s">
-        <v>100</v>
-      </c>
-      <c r="E37" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1077,10 +1092,10 @@
         <v>34</v>
       </c>
       <c r="B38" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C38" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -1088,10 +1103,10 @@
         <v>34</v>
       </c>
       <c r="B39" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C39" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
@@ -1099,21 +1114,24 @@
         <v>34</v>
       </c>
       <c r="B40" t="s">
-        <v>11</v>
+        <v>97</v>
       </c>
       <c r="C40" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>34</v>
-      </c>
-      <c r="B41" t="s">
-        <v>98</v>
-      </c>
-      <c r="C41" t="s">
-        <v>97</v>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>35</v>
+      </c>
+      <c r="B42" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" t="s">
+        <v>83</v>
+      </c>
+      <c r="D42" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
@@ -1121,24 +1139,27 @@
         <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C43" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>36</v>
+      </c>
+      <c r="B45" t="s">
+        <v>7</v>
+      </c>
+      <c r="C45" t="s">
         <v>84</v>
       </c>
-      <c r="D43" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>35</v>
-      </c>
-      <c r="B44" t="s">
-        <v>1</v>
-      </c>
-      <c r="C44" t="s">
-        <v>54</v>
+      <c r="D45" t="s">
+        <v>63</v>
+      </c>
+      <c r="E45" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
@@ -1146,16 +1167,10 @@
         <v>36</v>
       </c>
       <c r="B46" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C46" t="s">
-        <v>85</v>
-      </c>
-      <c r="D46" t="s">
-        <v>63</v>
-      </c>
-      <c r="E46" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -1163,10 +1178,10 @@
         <v>36</v>
       </c>
       <c r="B47" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C47" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -1174,142 +1189,142 @@
         <v>36</v>
       </c>
       <c r="B48" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C48" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>36</v>
-      </c>
-      <c r="B49" t="s">
-        <v>11</v>
-      </c>
-      <c r="C49" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
         <v>37</v>
       </c>
-      <c r="B51" t="s">
-        <v>74</v>
-      </c>
-      <c r="C51" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B50" t="s">
+        <v>73</v>
+      </c>
+      <c r="C50" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>12</v>
+      </c>
+      <c r="B52" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>12</v>
       </c>
       <c r="B53" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="C53" t="s">
+        <v>104</v>
+      </c>
+      <c r="D53" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>12</v>
       </c>
       <c r="B54" t="s">
-        <v>5</v>
-      </c>
-      <c r="C54" t="s">
-        <v>105</v>
-      </c>
-      <c r="D54" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+      <c r="E54" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>12</v>
       </c>
       <c r="B55" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C55" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>12</v>
       </c>
       <c r="B56" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C56" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>11</v>
+        <v>97</v>
       </c>
       <c r="C57" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C58" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>12</v>
       </c>
       <c r="B59" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C59" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>12</v>
-      </c>
-      <c r="B60" t="s">
         <v>103</v>
       </c>
-      <c r="C60" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>14</v>
+      </c>
+      <c r="B62" t="s">
+        <v>15</v>
+      </c>
+      <c r="C62" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>14</v>
       </c>
       <c r="B63" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C63" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>14</v>
       </c>
       <c r="B64" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C64" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
@@ -1317,21 +1332,24 @@
         <v>14</v>
       </c>
       <c r="B65" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C65" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
-        <v>14</v>
-      </c>
-      <c r="B66" t="s">
-        <v>16</v>
-      </c>
-      <c r="C66" t="s">
         <v>55</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>17</v>
+      </c>
+      <c r="B67" t="s">
+        <v>18</v>
+      </c>
+      <c r="C67" t="s">
+        <v>85</v>
+      </c>
+      <c r="E67" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
@@ -1339,13 +1357,13 @@
         <v>17</v>
       </c>
       <c r="B68" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C68" t="s">
-        <v>86</v>
+        <v>112</v>
       </c>
       <c r="E68" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
@@ -1353,13 +1371,10 @@
         <v>17</v>
       </c>
       <c r="B69" t="s">
-        <v>4</v>
-      </c>
-      <c r="C69" t="s">
-        <v>69</v>
+        <v>6</v>
       </c>
       <c r="E69" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.2">
@@ -1367,41 +1382,38 @@
         <v>17</v>
       </c>
       <c r="B70" t="s">
+        <v>9</v>
+      </c>
+      <c r="E70" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>38</v>
+      </c>
+      <c r="B72" t="s">
+        <v>91</v>
+      </c>
+      <c r="C72" t="s">
+        <v>89</v>
+      </c>
+      <c r="D72" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>19</v>
+      </c>
+      <c r="B74" t="s">
         <v>6</v>
       </c>
-      <c r="C70" t="s">
-        <v>50</v>
-      </c>
-      <c r="E70" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
-        <v>17</v>
-      </c>
-      <c r="B71" t="s">
-        <v>9</v>
-      </c>
-      <c r="C71" t="s">
-        <v>53</v>
-      </c>
-      <c r="E71" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
-        <v>38</v>
-      </c>
-      <c r="B73" t="s">
-        <v>92</v>
-      </c>
-      <c r="C73" t="s">
-        <v>90</v>
-      </c>
-      <c r="D73" t="s">
-        <v>91</v>
+      <c r="C74" t="s">
+        <v>79</v>
+      </c>
+      <c r="D74" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.2">
@@ -1409,13 +1421,7 @@
         <v>19</v>
       </c>
       <c r="B75" t="s">
-        <v>6</v>
-      </c>
-      <c r="C75" t="s">
-        <v>80</v>
-      </c>
-      <c r="D75" t="s">
-        <v>71</v>
+        <v>5</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -1423,7 +1429,10 @@
         <v>19</v>
       </c>
       <c r="B76" t="s">
-        <v>5</v>
+        <v>10</v>
+      </c>
+      <c r="C76" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
@@ -1431,10 +1440,10 @@
         <v>19</v>
       </c>
       <c r="B77" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C77" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
@@ -1442,10 +1451,10 @@
         <v>19</v>
       </c>
       <c r="B78" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C78" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -1453,10 +1462,10 @@
         <v>19</v>
       </c>
       <c r="B79" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C79" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
@@ -1464,10 +1473,10 @@
         <v>19</v>
       </c>
       <c r="B80" t="s">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="C80" t="s">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
@@ -1475,10 +1484,10 @@
         <v>19</v>
       </c>
       <c r="B81" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C81" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
@@ -1486,21 +1495,18 @@
         <v>19</v>
       </c>
       <c r="B82" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C82" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>19</v>
-      </c>
-      <c r="B83" t="s">
         <v>77</v>
       </c>
-      <c r="C83" t="s">
-        <v>78</v>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>20</v>
+      </c>
+      <c r="B84" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
@@ -1508,7 +1514,13 @@
         <v>20</v>
       </c>
       <c r="B85" t="s">
-        <v>21</v>
+        <v>8</v>
+      </c>
+      <c r="C85" t="s">
+        <v>78</v>
+      </c>
+      <c r="D85" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
@@ -1516,13 +1528,10 @@
         <v>20</v>
       </c>
       <c r="B86" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C86" t="s">
-        <v>79</v>
-      </c>
-      <c r="D86" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
@@ -1530,10 +1539,10 @@
         <v>20</v>
       </c>
       <c r="B87" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C87" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
@@ -1541,10 +1550,10 @@
         <v>20</v>
       </c>
       <c r="B88" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C88" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
@@ -1552,10 +1561,10 @@
         <v>20</v>
       </c>
       <c r="B89" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C89" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
@@ -1563,10 +1572,10 @@
         <v>20</v>
       </c>
       <c r="B90" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C90" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
@@ -1574,10 +1583,7 @@
         <v>20</v>
       </c>
       <c r="B91" t="s">
-        <v>11</v>
-      </c>
-      <c r="C91" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
@@ -1585,24 +1591,16 @@
         <v>20</v>
       </c>
       <c r="B92" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>20</v>
-      </c>
-      <c r="B93" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updates to general ODM v2/v3 ID code
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{854DE97F-5196-A44F-B2B6-C29DF46C9CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{337A8383-96CF-B74C-A2A8-D4C9F082941D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="110">
   <si>
     <t>addresses</t>
   </si>
@@ -365,15 +365,6 @@
   </si>
   <si>
     <t>True if (dat.contacts.firstName or dat.contacts.lastName or dat.contacts.email or dat.contacts.coPhone or dat.contacts.role) else ""</t>
-  </si>
-  <si>
-    <t>dat.contacts.get_first_linked_value("contactID", linkage_path="datasets_to_contacts_funderCont_contactID")</t>
-  </si>
-  <si>
-    <t>dat.contacts.get_first_linked_value("contactID", linkage_path="datasets_to_contacts_custodyCont_contactID")</t>
-  </si>
-  <si>
-    <t>dat.measures.get_first_linked_value("measureRepID", linkage_path="qualityReports_to_measures_measure")</t>
   </si>
 </sst>
 </file>
@@ -812,9 +803,6 @@
       <c r="B6" t="s">
         <v>2</v>
       </c>
-      <c r="C6" t="s">
-        <v>46</v>
-      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -887,9 +875,6 @@
       <c r="B16" t="s">
         <v>28</v>
       </c>
-      <c r="C16" t="s">
-        <v>110</v>
-      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
@@ -898,9 +883,6 @@
       <c r="B17" t="s">
         <v>29</v>
       </c>
-      <c r="C17" t="s">
-        <v>111</v>
-      </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
@@ -1358,9 +1340,6 @@
       </c>
       <c r="B68" t="s">
         <v>4</v>
-      </c>
-      <c r="C68" t="s">
-        <v>112</v>
       </c>
       <c r="E68" t="s">
         <v>56</v>

</xml_diff>

<commit_message>
Minor updates to ID code, changes to fn.datetimetz function
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{337A8383-96CF-B74C-A2A8-D4C9F082941D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE6EDF2E-86C7-9D4B-B40A-AD7779F3EF63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="122">
   <si>
     <t>addresses</t>
   </si>
@@ -253,24 +253,15 @@
     <t>fn.makeid(datEmpty.addresses.country, datEmpty.addresses.pCode, datEmpty.addresses.city[:3])</t>
   </si>
   <si>
-    <t>fn.datetimetz(dat.samples.__collDT.split('/!/'))</t>
-  </si>
-  <si>
     <t>protocolRelationshipsID</t>
   </si>
   <si>
     <t>collDTStart</t>
   </si>
   <si>
-    <t>fn.datetimetz(dat.samples.__collDTStart.split('/!/'))</t>
-  </si>
-  <si>
     <t>collDTEnd</t>
   </si>
   <si>
-    <t>fn.datetimetz(dat.samples.__collDTEnd.split('/!/'))</t>
-  </si>
-  <si>
     <t>fn.makeid(dat.sites.__siteID)</t>
   </si>
   <si>
@@ -365,6 +356,51 @@
   </si>
   <si>
     <t>True if (dat.contacts.firstName or dat.contacts.lastName or dat.contacts.email or dat.contacts.coPhone or dat.contacts.role) else ""</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.samples.__collDT, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.samples.__collDTStart, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.samples.__collDTEnd, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>reportDate</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.measures.__reportDate, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>aDateStart</t>
+  </si>
+  <si>
+    <t>aDateEnd</t>
+  </si>
+  <si>
+    <t>relDateStart</t>
+  </si>
+  <si>
+    <t>relDateEnd</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.measures.__aDateStart, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.measures.__aDateEnd, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.measures.__relDateStart, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.measures.__relDateEnd, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>epiWeekStart</t>
+  </si>
+  <si>
+    <t>fn.dateparse(dat.measures.__epiWeekStart)</t>
   </si>
 </sst>
 </file>
@@ -725,7 +761,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A1991E-0020-B448-B50F-72C1AC9C88C8}">
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E102"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -750,21 +786,21 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" t="s">
         <v>92</v>
-      </c>
-      <c r="B2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
@@ -787,7 +823,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D5" t="s">
         <v>71</v>
@@ -812,10 +848,10 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -834,10 +870,10 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
+        <v>103</v>
+      </c>
+      <c r="C10" t="s">
         <v>106</v>
-      </c>
-      <c r="C10" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -861,10 +897,10 @@
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D15" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E15" s="1"/>
     </row>
@@ -911,7 +947,7 @@
         <v>16</v>
       </c>
       <c r="C21" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D21" t="s">
         <v>59</v>
@@ -944,7 +980,7 @@
         <v>4</v>
       </c>
       <c r="C26" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D26" t="s">
         <v>60</v>
@@ -1041,217 +1077,217 @@
         <v>48</v>
       </c>
     </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>3</v>
+      </c>
+      <c r="B35" t="s">
+        <v>110</v>
+      </c>
+      <c r="C35" t="s">
+        <v>111</v>
+      </c>
+    </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>9</v>
+        <v>112</v>
       </c>
       <c r="C36" t="s">
-        <v>98</v>
-      </c>
-      <c r="D36" t="s">
-        <v>99</v>
-      </c>
-      <c r="E36" t="s">
-        <v>61</v>
+        <v>116</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B37" t="s">
-        <v>5</v>
+        <v>113</v>
       </c>
       <c r="C37" t="s">
-        <v>49</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B38" t="s">
-        <v>10</v>
+        <v>114</v>
       </c>
       <c r="C38" t="s">
-        <v>47</v>
+        <v>118</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B39" t="s">
-        <v>11</v>
+        <v>115</v>
       </c>
       <c r="C39" t="s">
-        <v>48</v>
+        <v>119</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B40" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="C40" t="s">
-        <v>96</v>
+        <v>121</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C42" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="D42" t="s">
-        <v>62</v>
+        <v>96</v>
+      </c>
+      <c r="E42" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B43" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C43" t="s">
-        <v>54</v>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>34</v>
+      </c>
+      <c r="B44" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B45" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C45" t="s">
-        <v>84</v>
-      </c>
-      <c r="D45" t="s">
-        <v>63</v>
-      </c>
-      <c r="E45" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B46" t="s">
-        <v>2</v>
+        <v>94</v>
       </c>
       <c r="C46" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>36</v>
-      </c>
-      <c r="B47" t="s">
-        <v>10</v>
-      </c>
-      <c r="C47" t="s">
-        <v>47</v>
+        <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
+        <v>35</v>
+      </c>
+      <c r="B48" t="s">
+        <v>10</v>
+      </c>
+      <c r="C48" t="s">
+        <v>80</v>
+      </c>
+      <c r="D48" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>35</v>
+      </c>
+      <c r="B49" t="s">
+        <v>1</v>
+      </c>
+      <c r="C49" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
         <v>36</v>
       </c>
-      <c r="B48" t="s">
-        <v>11</v>
-      </c>
-      <c r="C48" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>37</v>
-      </c>
-      <c r="B50" t="s">
-        <v>73</v>
-      </c>
-      <c r="C50" t="s">
-        <v>86</v>
+      <c r="B51" t="s">
+        <v>7</v>
+      </c>
+      <c r="C51" t="s">
+        <v>81</v>
+      </c>
+      <c r="D51" t="s">
+        <v>63</v>
+      </c>
+      <c r="E51" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="B52" t="s">
-        <v>13</v>
+        <v>2</v>
+      </c>
+      <c r="C52" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="B53" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C53" t="s">
-        <v>104</v>
-      </c>
-      <c r="D53" t="s">
-        <v>105</v>
+        <v>47</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="B54" t="s">
-        <v>2</v>
-      </c>
-      <c r="E54" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>12</v>
-      </c>
-      <c r="B55" t="s">
-        <v>10</v>
-      </c>
-      <c r="C55" t="s">
-        <v>47</v>
+        <v>11</v>
+      </c>
+      <c r="C54" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="B56" t="s">
-        <v>11</v>
+        <v>72</v>
       </c>
       <c r="C56" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
-        <v>12</v>
-      </c>
-      <c r="B57" t="s">
-        <v>97</v>
-      </c>
-      <c r="C57" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -1259,10 +1295,7 @@
         <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>100</v>
-      </c>
-      <c r="C58" t="s">
-        <v>101</v>
+        <v>13</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
@@ -1270,181 +1303,184 @@
         <v>12</v>
       </c>
       <c r="B59" t="s">
+        <v>5</v>
+      </c>
+      <c r="C59" t="s">
+        <v>101</v>
+      </c>
+      <c r="D59" t="s">
         <v>102</v>
       </c>
-      <c r="C59" t="s">
-        <v>103</v>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>12</v>
+      </c>
+      <c r="B60" t="s">
+        <v>2</v>
+      </c>
+      <c r="E60" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>12</v>
+      </c>
+      <c r="B61" t="s">
+        <v>10</v>
+      </c>
+      <c r="C61" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B62" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C62" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B63" t="s">
-        <v>10</v>
+        <v>94</v>
       </c>
       <c r="C63" t="s">
-        <v>47</v>
+        <v>93</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B64" t="s">
-        <v>11</v>
+        <v>97</v>
       </c>
       <c r="C64" t="s">
-        <v>48</v>
+        <v>98</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B65" t="s">
-        <v>16</v>
+        <v>99</v>
       </c>
       <c r="C65" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
-        <v>17</v>
-      </c>
-      <c r="B67" t="s">
-        <v>18</v>
-      </c>
-      <c r="C67" t="s">
-        <v>85</v>
-      </c>
-      <c r="E67" t="s">
-        <v>45</v>
+        <v>100</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B68" t="s">
-        <v>4</v>
-      </c>
-      <c r="E68" t="s">
-        <v>56</v>
+        <v>15</v>
+      </c>
+      <c r="C68" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B69" t="s">
-        <v>6</v>
-      </c>
-      <c r="E69" t="s">
-        <v>57</v>
+        <v>10</v>
+      </c>
+      <c r="C69" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
+        <v>14</v>
+      </c>
+      <c r="B70" t="s">
+        <v>11</v>
+      </c>
+      <c r="C70" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>14</v>
+      </c>
+      <c r="B71" t="s">
+        <v>16</v>
+      </c>
+      <c r="C71" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
         <v>17</v>
       </c>
-      <c r="B70" t="s">
-        <v>9</v>
-      </c>
-      <c r="E70" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
-        <v>38</v>
-      </c>
-      <c r="B72" t="s">
-        <v>91</v>
-      </c>
-      <c r="C72" t="s">
-        <v>89</v>
-      </c>
-      <c r="D72" t="s">
-        <v>90</v>
+      <c r="B73" t="s">
+        <v>18</v>
+      </c>
+      <c r="C73" t="s">
+        <v>82</v>
+      </c>
+      <c r="E73" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B74" t="s">
-        <v>6</v>
-      </c>
-      <c r="C74" t="s">
-        <v>79</v>
-      </c>
-      <c r="D74" t="s">
-        <v>70</v>
+        <v>4</v>
+      </c>
+      <c r="E74" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B75" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="E75" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B76" t="s">
-        <v>10</v>
-      </c>
-      <c r="C76" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
-        <v>19</v>
-      </c>
-      <c r="B77" t="s">
-        <v>11</v>
-      </c>
-      <c r="C77" t="s">
-        <v>48</v>
+        <v>9</v>
+      </c>
+      <c r="E76" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B78" t="s">
-        <v>8</v>
+        <v>88</v>
       </c>
       <c r="C78" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
-        <v>19</v>
-      </c>
-      <c r="B79" t="s">
-        <v>2</v>
-      </c>
-      <c r="C79" t="s">
-        <v>46</v>
+        <v>86</v>
+      </c>
+      <c r="D78" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
@@ -1452,10 +1488,13 @@
         <v>19</v>
       </c>
       <c r="B80" t="s">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="C80" t="s">
-        <v>72</v>
+        <v>76</v>
+      </c>
+      <c r="D80" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
@@ -1463,10 +1502,7 @@
         <v>19</v>
       </c>
       <c r="B81" t="s">
-        <v>74</v>
-      </c>
-      <c r="C81" t="s">
-        <v>75</v>
+        <v>5</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
@@ -1474,76 +1510,76 @@
         <v>19</v>
       </c>
       <c r="B82" t="s">
-        <v>76</v>
+        <v>10</v>
       </c>
       <c r="C82" t="s">
-        <v>77</v>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>19</v>
+      </c>
+      <c r="B83" t="s">
+        <v>11</v>
+      </c>
+      <c r="C83" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B84" t="s">
-        <v>21</v>
+        <v>8</v>
+      </c>
+      <c r="C84" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B85" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C85" t="s">
-        <v>78</v>
-      </c>
-      <c r="D85" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B86" t="s">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="C86" t="s">
-        <v>46</v>
+        <v>107</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B87" t="s">
-        <v>7</v>
+        <v>73</v>
       </c>
       <c r="C87" t="s">
-        <v>51</v>
+        <v>108</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B88" t="s">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="C88" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
-        <v>20</v>
-      </c>
-      <c r="B89" t="s">
-        <v>10</v>
-      </c>
-      <c r="C89" t="s">
-        <v>47</v>
+        <v>109</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
@@ -1551,10 +1587,7 @@
         <v>20</v>
       </c>
       <c r="B90" t="s">
-        <v>11</v>
-      </c>
-      <c r="C90" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
@@ -1562,7 +1595,13 @@
         <v>20</v>
       </c>
       <c r="B91" t="s">
-        <v>22</v>
+        <v>8</v>
+      </c>
+      <c r="C91" t="s">
+        <v>75</v>
+      </c>
+      <c r="D91" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
@@ -1570,16 +1609,79 @@
         <v>20</v>
       </c>
       <c r="B92" t="s">
-        <v>23</v>
+        <v>2</v>
+      </c>
+      <c r="C92" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>20</v>
+      </c>
+      <c r="B93" t="s">
+        <v>7</v>
+      </c>
+      <c r="C93" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>39</v>
+        <v>20</v>
+      </c>
+      <c r="B94" t="s">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>20</v>
+      </c>
+      <c r="B95" t="s">
+        <v>10</v>
+      </c>
+      <c r="C95" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
+        <v>20</v>
+      </c>
+      <c r="B96" t="s">
+        <v>11</v>
+      </c>
+      <c r="C96" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>20</v>
+      </c>
+      <c r="B97" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>20</v>
+      </c>
+      <c r="B98" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove datasetID from protocols, contacts, addresses
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE6EDF2E-86C7-9D4B-B40A-AD7779F3EF63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{726DD5F2-5980-634E-BF69-26D006AEA8BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="122">
   <si>
     <t>addresses</t>
   </si>
@@ -761,7 +761,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A1991E-0020-B448-B50F-72C1AC9C88C8}">
-  <dimension ref="A1:E102"/>
+  <dimension ref="A1:E100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -832,12 +832,18 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" t="s">
-        <v>2</v>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -845,13 +851,10 @@
         <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
-      </c>
-      <c r="D8" t="s">
-        <v>105</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -859,26 +862,23 @@
         <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>103</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" t="s">
-        <v>103</v>
-      </c>
-      <c r="C10" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -886,30 +886,30 @@
         <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C14" t="s">
+        <v>84</v>
+      </c>
+      <c r="D14" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" s="1"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>2</v>
-      </c>
-      <c r="C15" t="s">
-        <v>84</v>
-      </c>
-      <c r="D15" t="s">
-        <v>85</v>
-      </c>
-      <c r="E15" s="1"/>
+        <v>28</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -917,7 +917,7 @@
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -925,18 +925,27 @@
         <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" t="s">
         <v>31</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C18" t="s">
         <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E20" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -944,32 +953,32 @@
         <v>32</v>
       </c>
       <c r="B21" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>78</v>
-      </c>
-      <c r="D21" t="s">
-        <v>59</v>
-      </c>
-      <c r="E21" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>32</v>
-      </c>
-      <c r="B22" t="s">
-        <v>10</v>
-      </c>
-      <c r="C22" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" t="s">
+        <v>79</v>
+      </c>
+      <c r="D25" t="s">
+        <v>60</v>
+      </c>
+      <c r="E25" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -977,16 +986,10 @@
         <v>3</v>
       </c>
       <c r="B26" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>79</v>
-      </c>
-      <c r="D26" t="s">
-        <v>60</v>
-      </c>
-      <c r="E26" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -994,10 +997,10 @@
         <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -1005,10 +1008,10 @@
         <v>3</v>
       </c>
       <c r="B28" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C28" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -1016,10 +1019,10 @@
         <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C29" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -1027,10 +1030,10 @@
         <v>3</v>
       </c>
       <c r="B30" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C30" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1038,10 +1041,10 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C31" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -1049,10 +1052,10 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -1060,10 +1063,10 @@
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C33" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
@@ -1071,10 +1074,10 @@
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>11</v>
+        <v>110</v>
       </c>
       <c r="C34" t="s">
-        <v>48</v>
+        <v>111</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
@@ -1082,10 +1085,10 @@
         <v>3</v>
       </c>
       <c r="B35" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C35" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1093,10 +1096,10 @@
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C36" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1104,10 +1107,10 @@
         <v>3</v>
       </c>
       <c r="B37" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C37" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1115,10 +1118,10 @@
         <v>3</v>
       </c>
       <c r="B38" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C38" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -1126,21 +1129,27 @@
         <v>3</v>
       </c>
       <c r="B39" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C39" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>3</v>
-      </c>
-      <c r="B40" t="s">
-        <v>120</v>
-      </c>
-      <c r="C40" t="s">
         <v>121</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>34</v>
+      </c>
+      <c r="B41" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" t="s">
+        <v>95</v>
+      </c>
+      <c r="D41" t="s">
+        <v>96</v>
+      </c>
+      <c r="E41" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -1148,16 +1157,10 @@
         <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C42" t="s">
-        <v>95</v>
-      </c>
-      <c r="D42" t="s">
-        <v>96</v>
-      </c>
-      <c r="E42" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
@@ -1165,10 +1168,10 @@
         <v>34</v>
       </c>
       <c r="B43" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C43" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
@@ -1176,10 +1179,10 @@
         <v>34</v>
       </c>
       <c r="B44" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C44" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -1187,21 +1190,24 @@
         <v>34</v>
       </c>
       <c r="B45" t="s">
-        <v>11</v>
+        <v>94</v>
       </c>
       <c r="C45" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>34</v>
-      </c>
-      <c r="B46" t="s">
-        <v>94</v>
-      </c>
-      <c r="C46" t="s">
         <v>93</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>35</v>
+      </c>
+      <c r="B47" t="s">
+        <v>10</v>
+      </c>
+      <c r="C47" t="s">
+        <v>80</v>
+      </c>
+      <c r="D47" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -1209,24 +1215,27 @@
         <v>35</v>
       </c>
       <c r="B48" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>80</v>
-      </c>
-      <c r="D48" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>35</v>
-      </c>
-      <c r="B49" t="s">
-        <v>1</v>
-      </c>
-      <c r="C49" t="s">
         <v>54</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>36</v>
+      </c>
+      <c r="B50" t="s">
+        <v>7</v>
+      </c>
+      <c r="C50" t="s">
+        <v>81</v>
+      </c>
+      <c r="D50" t="s">
+        <v>63</v>
+      </c>
+      <c r="E50" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1234,16 +1243,10 @@
         <v>36</v>
       </c>
       <c r="B51" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C51" t="s">
-        <v>81</v>
-      </c>
-      <c r="D51" t="s">
-        <v>63</v>
-      </c>
-      <c r="E51" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
@@ -1251,10 +1254,10 @@
         <v>36</v>
       </c>
       <c r="B52" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C52" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
@@ -1262,32 +1265,29 @@
         <v>36</v>
       </c>
       <c r="B53" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C53" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>36</v>
-      </c>
-      <c r="B54" t="s">
-        <v>11</v>
-      </c>
-      <c r="C54" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
         <v>37</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B55" t="s">
         <v>72</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C55" t="s">
         <v>83</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>12</v>
+      </c>
+      <c r="B57" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -1295,7 +1295,13 @@
         <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>13</v>
+        <v>5</v>
+      </c>
+      <c r="C58" t="s">
+        <v>101</v>
+      </c>
+      <c r="D58" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
@@ -1303,13 +1309,10 @@
         <v>12</v>
       </c>
       <c r="B59" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C59" t="s">
-        <v>101</v>
-      </c>
-      <c r="D59" t="s">
-        <v>102</v>
+        <v>47</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.2">
@@ -1317,10 +1320,10 @@
         <v>12</v>
       </c>
       <c r="B60" t="s">
-        <v>2</v>
-      </c>
-      <c r="E60" t="s">
-        <v>46</v>
+        <v>11</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
@@ -1328,10 +1331,10 @@
         <v>12</v>
       </c>
       <c r="B61" t="s">
-        <v>10</v>
+        <v>94</v>
       </c>
       <c r="C61" t="s">
-        <v>47</v>
+        <v>93</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.2">
@@ -1339,10 +1342,10 @@
         <v>12</v>
       </c>
       <c r="B62" t="s">
-        <v>11</v>
+        <v>97</v>
       </c>
       <c r="C62" t="s">
-        <v>48</v>
+        <v>98</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
@@ -1350,32 +1353,32 @@
         <v>12</v>
       </c>
       <c r="B63" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C63" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
-        <v>12</v>
-      </c>
-      <c r="B64" t="s">
-        <v>97</v>
-      </c>
-      <c r="C64" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>12</v>
-      </c>
-      <c r="B65" t="s">
-        <v>99</v>
-      </c>
-      <c r="C65" t="s">
         <v>100</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>14</v>
+      </c>
+      <c r="B66" t="s">
+        <v>15</v>
+      </c>
+      <c r="C66" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>14</v>
+      </c>
+      <c r="B67" t="s">
+        <v>10</v>
+      </c>
+      <c r="C67" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
@@ -1383,10 +1386,10 @@
         <v>14</v>
       </c>
       <c r="B68" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C68" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
@@ -1394,32 +1397,35 @@
         <v>14</v>
       </c>
       <c r="B69" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C69" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
-        <v>14</v>
-      </c>
-      <c r="B70" t="s">
-        <v>11</v>
-      </c>
-      <c r="C70" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B71" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C71" t="s">
-        <v>55</v>
+        <v>82</v>
+      </c>
+      <c r="E71" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>17</v>
+      </c>
+      <c r="B72" t="s">
+        <v>4</v>
+      </c>
+      <c r="E72" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.2">
@@ -1427,13 +1433,10 @@
         <v>17</v>
       </c>
       <c r="B73" t="s">
-        <v>18</v>
-      </c>
-      <c r="C73" t="s">
-        <v>82</v>
+        <v>6</v>
       </c>
       <c r="E73" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
@@ -1441,46 +1444,46 @@
         <v>17</v>
       </c>
       <c r="B74" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E74" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
-        <v>17</v>
-      </c>
-      <c r="B75" t="s">
-        <v>6</v>
-      </c>
-      <c r="E75" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="B76" t="s">
-        <v>9</v>
-      </c>
-      <c r="E76" t="s">
-        <v>58</v>
+        <v>88</v>
+      </c>
+      <c r="C76" t="s">
+        <v>86</v>
+      </c>
+      <c r="D76" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="B78" t="s">
-        <v>88</v>
+        <v>6</v>
       </c>
       <c r="C78" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="D78" t="s">
-        <v>87</v>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>19</v>
+      </c>
+      <c r="B79" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
@@ -1488,13 +1491,10 @@
         <v>19</v>
       </c>
       <c r="B80" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C80" t="s">
-        <v>76</v>
-      </c>
-      <c r="D80" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
@@ -1502,7 +1502,10 @@
         <v>19</v>
       </c>
       <c r="B81" t="s">
-        <v>5</v>
+        <v>11</v>
+      </c>
+      <c r="C81" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
@@ -1510,10 +1513,10 @@
         <v>19</v>
       </c>
       <c r="B82" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C82" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
@@ -1521,10 +1524,10 @@
         <v>19</v>
       </c>
       <c r="B83" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="C83" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
@@ -1532,10 +1535,10 @@
         <v>19</v>
       </c>
       <c r="B84" t="s">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="C84" t="s">
-        <v>52</v>
+        <v>107</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
@@ -1543,10 +1546,10 @@
         <v>19</v>
       </c>
       <c r="B85" t="s">
-        <v>2</v>
+        <v>73</v>
       </c>
       <c r="C85" t="s">
-        <v>46</v>
+        <v>108</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
@@ -1554,32 +1557,32 @@
         <v>19</v>
       </c>
       <c r="B86" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C86" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
-        <v>19</v>
-      </c>
-      <c r="B87" t="s">
-        <v>73</v>
-      </c>
-      <c r="C87" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B88" t="s">
-        <v>74</v>
-      </c>
-      <c r="C88" t="s">
-        <v>109</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>20</v>
+      </c>
+      <c r="B89" t="s">
+        <v>8</v>
+      </c>
+      <c r="C89" t="s">
+        <v>75</v>
+      </c>
+      <c r="D89" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
@@ -1587,7 +1590,10 @@
         <v>20</v>
       </c>
       <c r="B90" t="s">
-        <v>21</v>
+        <v>2</v>
+      </c>
+      <c r="C90" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
@@ -1595,13 +1601,10 @@
         <v>20</v>
       </c>
       <c r="B91" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C91" t="s">
-        <v>75</v>
-      </c>
-      <c r="D91" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
@@ -1609,10 +1612,10 @@
         <v>20</v>
       </c>
       <c r="B92" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C92" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
@@ -1620,10 +1623,10 @@
         <v>20</v>
       </c>
       <c r="B93" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C93" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
@@ -1631,10 +1634,10 @@
         <v>20</v>
       </c>
       <c r="B94" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C94" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
@@ -1642,10 +1645,7 @@
         <v>20</v>
       </c>
       <c r="B95" t="s">
-        <v>10</v>
-      </c>
-      <c r="C95" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.2">
@@ -1653,35 +1653,16 @@
         <v>20</v>
       </c>
       <c r="B96" t="s">
-        <v>11</v>
-      </c>
-      <c r="C96" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
-        <v>20</v>
-      </c>
-      <c r="B97" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>20</v>
-      </c>
-      <c r="B98" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Replaced fn.dateparse with fn.date
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{726DD5F2-5980-634E-BF69-26D006AEA8BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF63358E-2FD9-0048-AA33-C5474D869E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -400,7 +400,7 @@
     <t>epiWeekStart</t>
   </si>
   <si>
-    <t>fn.dateparse(dat.measures.__epiWeekStart)</t>
+    <t>fn.date(dat.measures.__epiWeekStart)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
More complete general ID code, add code for all date and datetime slots for ODM
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF63358E-2FD9-0048-AA33-C5474D869E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F242D4A9-50C2-9B42-9EB4-C1E79B984EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="156">
   <si>
     <t>addresses</t>
   </si>
@@ -401,13 +401,115 @@
   </si>
   <si>
     <t>fn.date(dat.measures.__epiWeekStart)</t>
+  </si>
+  <si>
+    <t>datasetDate</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.datasets.__datasetDate, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>sentDate</t>
+  </si>
+  <si>
+    <t>recDate</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.samples.__sentDate, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.samples.__recDate, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>lastEdited</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.measures.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.qualityReports.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.accessions.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.protocolSteps.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.protocolRelationships.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>collDate</t>
+  </si>
+  <si>
+    <t>fn.date(dat.samples.__collDate)</t>
+  </si>
+  <si>
+    <t>fn.date(dat.samples.__epiWeekStart)</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.samples.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>polygonRelationships</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.polygonRelationships.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.organizations.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>calculations</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.calculations.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>phActions</t>
+  </si>
+  <si>
+    <t>actionDT</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.phActions.__actionDT, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.phActions.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.protocols.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.polygons.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.datasets.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.addresses.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.sampleRelationships.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.instruments.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.sites.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.contacts.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.datetimetz(dat.measureSets.__lastEdited, split_at='/!/')</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -422,6 +524,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -444,9 +552,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -761,7 +870,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A1991E-0020-B448-B50F-72C1AC9C88C8}">
-  <dimension ref="A1:E100"/>
+  <dimension ref="A1:E127"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -810,114 +919,111 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
+      <c r="A4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>0</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>1</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" t="s">
         <v>77</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D6" t="s">
         <v>71</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E6" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" t="s">
-        <v>11</v>
+        <v>0</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
-      </c>
-      <c r="D7" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" t="s">
-        <v>47</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>141</v>
       </c>
       <c r="B9" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>104</v>
+      </c>
+      <c r="D11" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" t="s">
-        <v>27</v>
+        <v>24</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C13" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="C14" t="s">
-        <v>84</v>
-      </c>
-      <c r="D14" t="s">
-        <v>85</v>
-      </c>
-      <c r="E14" s="1"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" t="s">
-        <v>28</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>26</v>
-      </c>
-      <c r="B16" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>26</v>
-      </c>
-      <c r="B17" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -925,137 +1031,123 @@
         <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>31</v>
-      </c>
-      <c r="C18" t="s">
-        <v>47</v>
-      </c>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" t="s">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19" t="s">
+        <v>85</v>
+      </c>
+      <c r="E19" s="1"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B20" t="s">
-        <v>16</v>
-      </c>
-      <c r="C20" t="s">
-        <v>78</v>
-      </c>
-      <c r="D20" t="s">
-        <v>59</v>
-      </c>
-      <c r="E20" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>10</v>
-      </c>
-      <c r="C21" t="s">
-        <v>47</v>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>33</v>
+        <v>26</v>
+      </c>
+      <c r="B23" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C24" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>3</v>
-      </c>
-      <c r="B25" t="s">
-        <v>4</v>
+        <v>26</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="C25" t="s">
-        <v>79</v>
-      </c>
-      <c r="D25" t="s">
-        <v>60</v>
-      </c>
-      <c r="E25" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>3</v>
-      </c>
-      <c r="B26" t="s">
-        <v>5</v>
-      </c>
-      <c r="C26" t="s">
-        <v>49</v>
+        <v>149</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C27" t="s">
-        <v>50</v>
+        <v>78</v>
+      </c>
+      <c r="D27" t="s">
+        <v>59</v>
+      </c>
+      <c r="E27" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C28" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>3</v>
-      </c>
-      <c r="B29" t="s">
-        <v>8</v>
+        <v>32</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="C29" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>3</v>
-      </c>
-      <c r="B30" t="s">
-        <v>2</v>
-      </c>
-      <c r="C30" t="s">
-        <v>46</v>
+        <v>152</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" t="s">
-        <v>9</v>
-      </c>
-      <c r="C31" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>3</v>
-      </c>
-      <c r="B32" t="s">
-        <v>10</v>
-      </c>
-      <c r="C32" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -1063,10 +1155,16 @@
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C33" t="s">
-        <v>48</v>
+        <v>79</v>
+      </c>
+      <c r="D33" t="s">
+        <v>60</v>
+      </c>
+      <c r="E33" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
@@ -1074,10 +1172,10 @@
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>110</v>
+        <v>5</v>
       </c>
       <c r="C34" t="s">
-        <v>111</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
@@ -1085,10 +1183,10 @@
         <v>3</v>
       </c>
       <c r="B35" t="s">
-        <v>112</v>
+        <v>6</v>
       </c>
       <c r="C35" t="s">
-        <v>116</v>
+        <v>50</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1096,10 +1194,10 @@
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>113</v>
+        <v>7</v>
       </c>
       <c r="C36" t="s">
-        <v>117</v>
+        <v>51</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1107,10 +1205,10 @@
         <v>3</v>
       </c>
       <c r="B37" t="s">
-        <v>114</v>
+        <v>8</v>
       </c>
       <c r="C37" t="s">
-        <v>118</v>
+        <v>52</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1118,10 +1216,10 @@
         <v>3</v>
       </c>
       <c r="B38" t="s">
-        <v>115</v>
+        <v>2</v>
       </c>
       <c r="C38" t="s">
-        <v>119</v>
+        <v>46</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -1129,129 +1227,142 @@
         <v>3</v>
       </c>
       <c r="B39" t="s">
-        <v>120</v>
+        <v>9</v>
       </c>
       <c r="C39" t="s">
-        <v>121</v>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>3</v>
+      </c>
+      <c r="B40" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B41" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C41" t="s">
-        <v>95</v>
-      </c>
-      <c r="D41" t="s">
-        <v>96</v>
-      </c>
-      <c r="E41" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B42" t="s">
-        <v>5</v>
+        <v>110</v>
       </c>
       <c r="C42" t="s">
-        <v>49</v>
+        <v>111</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B43" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="C43" t="s">
-        <v>47</v>
+        <v>116</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B44" t="s">
-        <v>11</v>
+        <v>113</v>
       </c>
       <c r="C44" t="s">
-        <v>48</v>
+        <v>117</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B45" t="s">
-        <v>94</v>
+        <v>114</v>
       </c>
       <c r="C45" t="s">
-        <v>93</v>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>3</v>
+      </c>
+      <c r="B46" t="s">
+        <v>115</v>
+      </c>
+      <c r="C46" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="B47" t="s">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="C47" t="s">
-        <v>80</v>
-      </c>
-      <c r="D47" t="s">
-        <v>62</v>
+        <v>121</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="B48" t="s">
-        <v>1</v>
+        <v>128</v>
       </c>
       <c r="C48" t="s">
-        <v>54</v>
+        <v>129</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B50" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C50" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="D50" t="s">
-        <v>63</v>
+        <v>96</v>
       </c>
       <c r="E50" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B51" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C51" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B52" t="s">
         <v>10</v>
@@ -1262,7 +1373,7 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B53" t="s">
         <v>11</v>
@@ -1271,398 +1382,671 @@
         <v>48</v>
       </c>
     </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>34</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C54" t="s">
+        <v>155</v>
+      </c>
+    </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B55" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="C55" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="B57" t="s">
-        <v>13</v>
+        <v>10</v>
+      </c>
+      <c r="C57" t="s">
+        <v>80</v>
+      </c>
+      <c r="D57" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="B58" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C58" t="s">
-        <v>101</v>
-      </c>
-      <c r="D58" t="s">
-        <v>102</v>
+        <v>54</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="B59" t="s">
-        <v>10</v>
+        <v>128</v>
       </c>
       <c r="C59" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>12</v>
-      </c>
-      <c r="B60" t="s">
-        <v>11</v>
-      </c>
-      <c r="C60" t="s">
-        <v>48</v>
+        <v>140</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>12</v>
+        <v>143</v>
       </c>
       <c r="B61" t="s">
-        <v>94</v>
+        <v>144</v>
       </c>
       <c r="C61" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
+        <v>143</v>
+      </c>
+      <c r="B62" t="s">
+        <v>128</v>
+      </c>
+      <c r="C62" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>36</v>
+      </c>
+      <c r="B64" t="s">
+        <v>7</v>
+      </c>
+      <c r="C64" t="s">
+        <v>81</v>
+      </c>
+      <c r="D64" t="s">
+        <v>63</v>
+      </c>
+      <c r="E64" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>36</v>
+      </c>
+      <c r="B65" t="s">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>36</v>
+      </c>
+      <c r="B66" t="s">
+        <v>10</v>
+      </c>
+      <c r="C66" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>36</v>
+      </c>
+      <c r="B67" t="s">
+        <v>11</v>
+      </c>
+      <c r="C67" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>36</v>
+      </c>
+      <c r="B68" t="s">
+        <v>128</v>
+      </c>
+      <c r="C68" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>138</v>
+      </c>
+      <c r="B70" t="s">
+        <v>128</v>
+      </c>
+      <c r="C70" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>37</v>
+      </c>
+      <c r="B72" t="s">
+        <v>72</v>
+      </c>
+      <c r="C72" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>37</v>
+      </c>
+      <c r="B73" t="s">
+        <v>128</v>
+      </c>
+      <c r="C73" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
         <v>12</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B75" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>12</v>
+      </c>
+      <c r="B76" t="s">
+        <v>5</v>
+      </c>
+      <c r="C76" t="s">
+        <v>101</v>
+      </c>
+      <c r="D76" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>12</v>
+      </c>
+      <c r="B77" t="s">
+        <v>10</v>
+      </c>
+      <c r="C77" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>12</v>
+      </c>
+      <c r="B78" t="s">
+        <v>11</v>
+      </c>
+      <c r="C78" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>12</v>
+      </c>
+      <c r="B79" t="s">
+        <v>128</v>
+      </c>
+      <c r="C79" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>12</v>
+      </c>
+      <c r="B80" t="s">
+        <v>94</v>
+      </c>
+      <c r="C80" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>12</v>
+      </c>
+      <c r="B81" t="s">
         <v>97</v>
       </c>
-      <c r="C62" t="s">
+      <c r="C81" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
         <v>12</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B82" t="s">
         <v>99</v>
       </c>
-      <c r="C63" t="s">
+      <c r="C82" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
         <v>14</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B84" t="s">
         <v>15</v>
       </c>
-      <c r="C66" t="s">
+      <c r="C84" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
         <v>14</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B85" t="s">
         <v>10</v>
       </c>
-      <c r="C67" t="s">
+      <c r="C85" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
         <v>14</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B86" t="s">
         <v>11</v>
       </c>
-      <c r="C68" t="s">
+      <c r="C86" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
         <v>14</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B87" t="s">
         <v>16</v>
       </c>
-      <c r="C69" t="s">
+      <c r="C87" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>14</v>
+      </c>
+      <c r="B88" t="s">
+        <v>128</v>
+      </c>
+      <c r="C88" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
         <v>17</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B90" t="s">
         <v>18</v>
       </c>
-      <c r="C71" t="s">
+      <c r="C90" t="s">
         <v>82</v>
       </c>
-      <c r="E71" t="s">
+      <c r="E90" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
         <v>17</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B91" t="s">
         <v>4</v>
       </c>
-      <c r="E72" t="s">
+      <c r="E91" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
         <v>17</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B92" t="s">
         <v>6</v>
       </c>
-      <c r="E73" t="s">
+      <c r="E92" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
         <v>17</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B93" t="s">
         <v>9</v>
       </c>
-      <c r="E74" t="s">
+      <c r="E93" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>17</v>
+      </c>
+      <c r="B94" t="s">
+        <v>128</v>
+      </c>
+      <c r="C94" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
         <v>38</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B96" t="s">
         <v>88</v>
       </c>
-      <c r="C76" t="s">
+      <c r="C96" t="s">
         <v>86</v>
       </c>
-      <c r="D76" t="s">
+      <c r="D96" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>38</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C97" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
         <v>19</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B99" t="s">
         <v>6</v>
       </c>
-      <c r="C78" t="s">
+      <c r="C99" t="s">
         <v>76</v>
       </c>
-      <c r="D78" t="s">
+      <c r="D99" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
         <v>19</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B100" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
         <v>19</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B101" t="s">
         <v>10</v>
       </c>
-      <c r="C80" t="s">
+      <c r="C101" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
         <v>19</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B102" t="s">
         <v>11</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C102" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
         <v>19</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B103" t="s">
         <v>8</v>
       </c>
-      <c r="C82" t="s">
+      <c r="C103" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
         <v>19</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B104" t="s">
         <v>2</v>
       </c>
-      <c r="C83" t="s">
+      <c r="C104" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
         <v>19</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B105" t="s">
         <v>68</v>
       </c>
-      <c r="C84" t="s">
+      <c r="C105" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
         <v>19</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B106" t="s">
         <v>73</v>
       </c>
-      <c r="C85" t="s">
+      <c r="C106" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
         <v>19</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B107" t="s">
         <v>74</v>
       </c>
-      <c r="C86" t="s">
+      <c r="C107" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>19</v>
+      </c>
+      <c r="B108" t="s">
+        <v>134</v>
+      </c>
+      <c r="C108" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>19</v>
+      </c>
+      <c r="B109" t="s">
+        <v>124</v>
+      </c>
+      <c r="C109" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>19</v>
+      </c>
+      <c r="B110" t="s">
+        <v>125</v>
+      </c>
+      <c r="C110" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>19</v>
+      </c>
+      <c r="B111" t="s">
+        <v>120</v>
+      </c>
+      <c r="C111" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>19</v>
+      </c>
+      <c r="B112" t="s">
+        <v>128</v>
+      </c>
+      <c r="C112" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
         <v>20</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B114" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
         <v>20</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B115" t="s">
         <v>8</v>
       </c>
-      <c r="C89" t="s">
+      <c r="C115" t="s">
         <v>75</v>
       </c>
-      <c r="D89" t="s">
+      <c r="D115" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
         <v>20</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B116" t="s">
         <v>2</v>
       </c>
-      <c r="C90" t="s">
+      <c r="C116" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
         <v>20</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B117" t="s">
         <v>7</v>
       </c>
-      <c r="C91" t="s">
+      <c r="C117" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
         <v>20</v>
       </c>
-      <c r="B92" t="s">
+      <c r="B118" t="s">
         <v>1</v>
       </c>
-      <c r="C92" t="s">
+      <c r="C118" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
         <v>20</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B119" t="s">
         <v>10</v>
       </c>
-      <c r="C93" t="s">
+      <c r="C119" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
         <v>20</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B120" t="s">
         <v>11</v>
       </c>
-      <c r="C94" t="s">
+      <c r="C120" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
         <v>20</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B121" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
         <v>20</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B122" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A123" t="s">
+        <v>20</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C123" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Minor updates to ID code
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F242D4A9-50C2-9B42-9EB4-C1E79B984EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2A7A57F-2E9E-5A4D-AE7E-84BB43378644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="156">
   <si>
     <t>addresses</t>
   </si>
@@ -870,7 +870,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A1991E-0020-B448-B50F-72C1AC9C88C8}">
-  <dimension ref="A1:E127"/>
+  <dimension ref="A1:E126"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -1127,209 +1127,215 @@
       <c r="A28" t="s">
         <v>32</v>
       </c>
-      <c r="B28" t="s">
-        <v>10</v>
+      <c r="B28" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="C28" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>32</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="C29" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B32" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" t="s">
+        <v>79</v>
+      </c>
+      <c r="D32" t="s">
+        <v>60</v>
+      </c>
+      <c r="E32" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C33" t="s">
-        <v>79</v>
-      </c>
-      <c r="D33" t="s">
-        <v>60</v>
-      </c>
-      <c r="E33" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C34" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>3</v>
       </c>
       <c r="B35" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C35" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C36" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>3</v>
       </c>
       <c r="B37" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C37" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>3</v>
       </c>
       <c r="B38" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C38" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>3</v>
       </c>
       <c r="B39" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>3</v>
       </c>
       <c r="B40" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C40" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>3</v>
       </c>
       <c r="B41" t="s">
-        <v>11</v>
+        <v>110</v>
       </c>
       <c r="C41" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>3</v>
       </c>
       <c r="B42" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C42" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>3</v>
       </c>
       <c r="B43" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C43" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>3</v>
       </c>
       <c r="B44" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C44" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>3</v>
       </c>
       <c r="B45" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C45" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>3</v>
       </c>
       <c r="B46" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C46" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>3</v>
       </c>
       <c r="B47" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="C47" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>3</v>
-      </c>
-      <c r="B48" t="s">
-        <v>128</v>
-      </c>
-      <c r="C48" t="s">
         <v>129</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>34</v>
+      </c>
+      <c r="B49" t="s">
+        <v>9</v>
+      </c>
+      <c r="C49" t="s">
+        <v>95</v>
+      </c>
+      <c r="D49" t="s">
+        <v>96</v>
+      </c>
+      <c r="E49" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1337,16 +1343,10 @@
         <v>34</v>
       </c>
       <c r="B50" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C50" t="s">
-        <v>95</v>
-      </c>
-      <c r="D50" t="s">
-        <v>96</v>
-      </c>
-      <c r="E50" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1354,10 +1354,10 @@
         <v>34</v>
       </c>
       <c r="B51" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C51" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
@@ -1365,43 +1365,46 @@
         <v>34</v>
       </c>
       <c r="B52" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C52" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>34</v>
       </c>
-      <c r="B53" t="s">
-        <v>11</v>
+      <c r="B53" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="C53" t="s">
-        <v>48</v>
+        <v>155</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>34</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>128</v>
+      <c r="B54" t="s">
+        <v>94</v>
       </c>
       <c r="C54" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>34</v>
-      </c>
-      <c r="B55" t="s">
-        <v>94</v>
-      </c>
-      <c r="C55" t="s">
         <v>93</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>35</v>
+      </c>
+      <c r="B56" t="s">
+        <v>10</v>
+      </c>
+      <c r="C56" t="s">
+        <v>80</v>
+      </c>
+      <c r="D56" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
@@ -1409,13 +1412,10 @@
         <v>35</v>
       </c>
       <c r="B57" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>80</v>
-      </c>
-      <c r="D57" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -1423,21 +1423,21 @@
         <v>35</v>
       </c>
       <c r="B58" t="s">
-        <v>1</v>
+        <v>128</v>
       </c>
       <c r="C58" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
-        <v>35</v>
-      </c>
-      <c r="B59" t="s">
-        <v>128</v>
-      </c>
-      <c r="C59" t="s">
         <v>140</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>143</v>
+      </c>
+      <c r="B60" t="s">
+        <v>144</v>
+      </c>
+      <c r="C60" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
@@ -1445,21 +1445,27 @@
         <v>143</v>
       </c>
       <c r="B61" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="C61" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>143</v>
-      </c>
-      <c r="B62" t="s">
-        <v>128</v>
-      </c>
-      <c r="C62" t="s">
         <v>146</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>36</v>
+      </c>
+      <c r="B63" t="s">
+        <v>7</v>
+      </c>
+      <c r="C63" t="s">
+        <v>81</v>
+      </c>
+      <c r="D63" t="s">
+        <v>63</v>
+      </c>
+      <c r="E63" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.2">
@@ -1467,16 +1473,10 @@
         <v>36</v>
       </c>
       <c r="B64" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C64" t="s">
-        <v>81</v>
-      </c>
-      <c r="D64" t="s">
-        <v>63</v>
-      </c>
-      <c r="E64" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
@@ -1484,10 +1484,10 @@
         <v>36</v>
       </c>
       <c r="B65" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C65" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
@@ -1495,10 +1495,10 @@
         <v>36</v>
       </c>
       <c r="B66" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C66" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
@@ -1506,32 +1506,32 @@
         <v>36</v>
       </c>
       <c r="B67" t="s">
-        <v>11</v>
+        <v>128</v>
       </c>
       <c r="C67" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
-        <v>36</v>
-      </c>
-      <c r="B68" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>138</v>
+      </c>
+      <c r="B69" t="s">
         <v>128</v>
       </c>
-      <c r="C68" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
-        <v>138</v>
-      </c>
-      <c r="B70" t="s">
-        <v>128</v>
-      </c>
-      <c r="C70" t="s">
+      <c r="C69" t="s">
         <v>139</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>37</v>
+      </c>
+      <c r="B71" t="s">
+        <v>72</v>
+      </c>
+      <c r="C71" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
@@ -1539,21 +1539,18 @@
         <v>37</v>
       </c>
       <c r="B72" t="s">
-        <v>72</v>
+        <v>128</v>
       </c>
       <c r="C72" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
-        <v>37</v>
-      </c>
-      <c r="B73" t="s">
-        <v>128</v>
-      </c>
-      <c r="C73" t="s">
         <v>133</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>12</v>
+      </c>
+      <c r="B74" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
@@ -1561,7 +1558,13 @@
         <v>12</v>
       </c>
       <c r="B75" t="s">
-        <v>13</v>
+        <v>5</v>
+      </c>
+      <c r="C75" t="s">
+        <v>101</v>
+      </c>
+      <c r="D75" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
@@ -1569,13 +1572,10 @@
         <v>12</v>
       </c>
       <c r="B76" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C76" t="s">
-        <v>101</v>
-      </c>
-      <c r="D76" t="s">
-        <v>102</v>
+        <v>47</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
@@ -1583,10 +1583,10 @@
         <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C77" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
@@ -1594,10 +1594,10 @@
         <v>12</v>
       </c>
       <c r="B78" t="s">
-        <v>11</v>
+        <v>128</v>
       </c>
       <c r="C78" t="s">
-        <v>48</v>
+        <v>147</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
@@ -1605,10 +1605,10 @@
         <v>12</v>
       </c>
       <c r="B79" t="s">
-        <v>128</v>
+        <v>94</v>
       </c>
       <c r="C79" t="s">
-        <v>147</v>
+        <v>93</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
@@ -1616,10 +1616,10 @@
         <v>12</v>
       </c>
       <c r="B80" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C80" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -1627,21 +1627,21 @@
         <v>12</v>
       </c>
       <c r="B81" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C81" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>12</v>
-      </c>
-      <c r="B82" t="s">
-        <v>99</v>
-      </c>
-      <c r="C82" t="s">
         <v>100</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>14</v>
+      </c>
+      <c r="B83" t="s">
+        <v>15</v>
+      </c>
+      <c r="C83" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
@@ -1649,10 +1649,10 @@
         <v>14</v>
       </c>
       <c r="B84" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C84" t="s">
-        <v>69</v>
+        <v>47</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
@@ -1660,10 +1660,10 @@
         <v>14</v>
       </c>
       <c r="B85" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C85" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.2">
@@ -1671,10 +1671,10 @@
         <v>14</v>
       </c>
       <c r="B86" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C86" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
@@ -1682,21 +1682,24 @@
         <v>14</v>
       </c>
       <c r="B87" t="s">
-        <v>16</v>
+        <v>128</v>
       </c>
       <c r="C87" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
-        <v>14</v>
-      </c>
-      <c r="B88" t="s">
-        <v>128</v>
-      </c>
-      <c r="C88" t="s">
         <v>132</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>17</v>
+      </c>
+      <c r="B89" t="s">
+        <v>18</v>
+      </c>
+      <c r="C89" t="s">
+        <v>82</v>
+      </c>
+      <c r="E89" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
@@ -1704,13 +1707,10 @@
         <v>17</v>
       </c>
       <c r="B90" t="s">
-        <v>18</v>
-      </c>
-      <c r="C90" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="E90" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
@@ -1718,10 +1718,10 @@
         <v>17</v>
       </c>
       <c r="B91" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E91" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
@@ -1729,10 +1729,10 @@
         <v>17</v>
       </c>
       <c r="B92" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E92" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
@@ -1740,46 +1740,49 @@
         <v>17</v>
       </c>
       <c r="B93" t="s">
-        <v>9</v>
-      </c>
-      <c r="E93" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
-        <v>17</v>
-      </c>
-      <c r="B94" t="s">
         <v>128</v>
       </c>
-      <c r="C94" t="s">
+      <c r="C93" t="s">
         <v>130</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>38</v>
+      </c>
+      <c r="B95" t="s">
+        <v>88</v>
+      </c>
+      <c r="C95" t="s">
+        <v>86</v>
+      </c>
+      <c r="D95" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>38</v>
       </c>
-      <c r="B96" t="s">
-        <v>88</v>
+      <c r="B96" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="C96" t="s">
-        <v>86</v>
-      </c>
-      <c r="D96" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
-        <v>38</v>
-      </c>
-      <c r="B97" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="C97" t="s">
         <v>151</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>19</v>
+      </c>
+      <c r="B98" t="s">
+        <v>6</v>
+      </c>
+      <c r="C98" t="s">
+        <v>76</v>
+      </c>
+      <c r="D98" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
@@ -1787,13 +1790,7 @@
         <v>19</v>
       </c>
       <c r="B99" t="s">
-        <v>6</v>
-      </c>
-      <c r="C99" t="s">
-        <v>76</v>
-      </c>
-      <c r="D99" t="s">
-        <v>70</v>
+        <v>5</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.2">
@@ -1801,7 +1798,10 @@
         <v>19</v>
       </c>
       <c r="B100" t="s">
-        <v>5</v>
+        <v>10</v>
+      </c>
+      <c r="C100" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.2">
@@ -1809,10 +1809,10 @@
         <v>19</v>
       </c>
       <c r="B101" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C101" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.2">
@@ -1820,10 +1820,10 @@
         <v>19</v>
       </c>
       <c r="B102" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C102" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.2">
@@ -1831,10 +1831,10 @@
         <v>19</v>
       </c>
       <c r="B103" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C103" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.2">
@@ -1842,10 +1842,10 @@
         <v>19</v>
       </c>
       <c r="B104" t="s">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="C104" t="s">
-        <v>46</v>
+        <v>107</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.2">
@@ -1853,10 +1853,10 @@
         <v>19</v>
       </c>
       <c r="B105" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C105" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.2">
@@ -1864,10 +1864,10 @@
         <v>19</v>
       </c>
       <c r="B106" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C106" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.2">
@@ -1875,10 +1875,10 @@
         <v>19</v>
       </c>
       <c r="B107" t="s">
-        <v>74</v>
+        <v>134</v>
       </c>
       <c r="C107" t="s">
-        <v>109</v>
+        <v>135</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
@@ -1886,10 +1886,10 @@
         <v>19</v>
       </c>
       <c r="B108" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="C108" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.2">
@@ -1897,10 +1897,10 @@
         <v>19</v>
       </c>
       <c r="B109" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C109" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.2">
@@ -1908,10 +1908,10 @@
         <v>19</v>
       </c>
       <c r="B110" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C110" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.2">
@@ -1919,21 +1919,18 @@
         <v>19</v>
       </c>
       <c r="B111" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="C111" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A112" t="s">
-        <v>19</v>
-      </c>
-      <c r="B112" t="s">
-        <v>128</v>
-      </c>
-      <c r="C112" t="s">
         <v>137</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>20</v>
+      </c>
+      <c r="B113" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.2">
@@ -1941,7 +1938,13 @@
         <v>20</v>
       </c>
       <c r="B114" t="s">
-        <v>21</v>
+        <v>8</v>
+      </c>
+      <c r="C114" t="s">
+        <v>75</v>
+      </c>
+      <c r="D114" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.2">
@@ -1949,13 +1952,10 @@
         <v>20</v>
       </c>
       <c r="B115" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C115" t="s">
-        <v>75</v>
-      </c>
-      <c r="D115" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.2">
@@ -1963,10 +1963,10 @@
         <v>20</v>
       </c>
       <c r="B116" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C116" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.2">
@@ -1974,10 +1974,10 @@
         <v>20</v>
       </c>
       <c r="B117" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C117" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.2">
@@ -1985,10 +1985,10 @@
         <v>20</v>
       </c>
       <c r="B118" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C118" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.2">
@@ -1996,10 +1996,10 @@
         <v>20</v>
       </c>
       <c r="B119" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C119" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.2">
@@ -2007,10 +2007,7 @@
         <v>20</v>
       </c>
       <c r="B120" t="s">
-        <v>11</v>
-      </c>
-      <c r="C120" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.2">
@@ -2018,35 +2015,27 @@
         <v>20</v>
       </c>
       <c r="B121" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>20</v>
       </c>
-      <c r="B122" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A123" t="s">
-        <v>20</v>
-      </c>
-      <c r="B123" s="2" t="s">
+      <c r="B122" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C123" t="s">
+      <c r="C122" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A125" t="s">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A124" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A127" t="s">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Use datEmpty instead of dat for generating qualityReportID
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2A7A57F-2E9E-5A4D-AE7E-84BB43378644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{753ECD02-B6DD-8845-82F2-8D695D444503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -283,9 +283,6 @@
     <t>fn.makeid(dat.polygons.__polygonID)</t>
   </si>
   <si>
-    <t>fn.makeid(datEmpty.qualityReports.qualityFlag, dat.qualityReports.measureRepID, dat.qualityReports.sampleID, dat.qualityReports.measureSetRepID)</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.protocolRelationships.protocolIDContainer, datEmpty.protocolRelationships.stepIDObj, datEmpty.protocolRelationships.relationshipID)</t>
   </si>
   <si>
@@ -503,6 +500,9 @@
   </si>
   <si>
     <t>fn.datetimetz(dat.measureSets.__lastEdited, split_at='/!/')</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.qualityReports.qualityFlag, datEmpty.qualityReports.measureRepID, datEmpty.qualityReports.sampleID, datEmpty.qualityReports.measureSetRepID)</t>
   </si>
 </sst>
 </file>
@@ -895,21 +895,21 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" t="s">
         <v>89</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>90</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>91</v>
-      </c>
-      <c r="D2" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
@@ -920,13 +920,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -957,21 +957,21 @@
         <v>0</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B9" t="s">
+        <v>127</v>
+      </c>
+      <c r="C9" t="s">
         <v>141</v>
-      </c>
-      <c r="B9" t="s">
-        <v>128</v>
-      </c>
-      <c r="C9" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -982,10 +982,10 @@
         <v>11</v>
       </c>
       <c r="C11" t="s">
+        <v>103</v>
+      </c>
+      <c r="D11" t="s">
         <v>104</v>
-      </c>
-      <c r="D11" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -1004,10 +1004,10 @@
         <v>24</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -1015,10 +1015,10 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -1042,10 +1042,10 @@
         <v>2</v>
       </c>
       <c r="C19" t="s">
+        <v>83</v>
+      </c>
+      <c r="D19" t="s">
         <v>84</v>
-      </c>
-      <c r="D19" t="s">
-        <v>85</v>
       </c>
       <c r="E19" s="1"/>
     </row>
@@ -1089,10 +1089,10 @@
         <v>26</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C24" t="s">
         <v>122</v>
-      </c>
-      <c r="C24" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
@@ -1100,10 +1100,10 @@
         <v>26</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C25" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -1128,10 +1128,10 @@
         <v>32</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C28" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -1249,10 +1249,10 @@
         <v>3</v>
       </c>
       <c r="B41" t="s">
+        <v>109</v>
+      </c>
+      <c r="C41" t="s">
         <v>110</v>
-      </c>
-      <c r="C41" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -1260,10 +1260,10 @@
         <v>3</v>
       </c>
       <c r="B42" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C42" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -1271,10 +1271,10 @@
         <v>3</v>
       </c>
       <c r="B43" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C43" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -1282,10 +1282,10 @@
         <v>3</v>
       </c>
       <c r="B44" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C44" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -1293,10 +1293,10 @@
         <v>3</v>
       </c>
       <c r="B45" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C45" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
@@ -1304,10 +1304,10 @@
         <v>3</v>
       </c>
       <c r="B46" t="s">
+        <v>119</v>
+      </c>
+      <c r="C46" t="s">
         <v>120</v>
-      </c>
-      <c r="C46" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -1315,10 +1315,10 @@
         <v>3</v>
       </c>
       <c r="B47" t="s">
+        <v>127</v>
+      </c>
+      <c r="C47" t="s">
         <v>128</v>
-      </c>
-      <c r="C47" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -1329,10 +1329,10 @@
         <v>9</v>
       </c>
       <c r="C49" t="s">
+        <v>94</v>
+      </c>
+      <c r="D49" t="s">
         <v>95</v>
-      </c>
-      <c r="D49" t="s">
-        <v>96</v>
       </c>
       <c r="E49" t="s">
         <v>61</v>
@@ -1376,10 +1376,10 @@
         <v>34</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C53" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
@@ -1387,10 +1387,10 @@
         <v>34</v>
       </c>
       <c r="B54" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C54" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
@@ -1423,32 +1423,32 @@
         <v>35</v>
       </c>
       <c r="B58" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C58" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
+        <v>142</v>
+      </c>
+      <c r="B60" t="s">
         <v>143</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C60" t="s">
         <v>144</v>
-      </c>
-      <c r="C60" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B61" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C61" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
@@ -1506,21 +1506,21 @@
         <v>36</v>
       </c>
       <c r="B67" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C67" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
+        <v>137</v>
+      </c>
+      <c r="B69" t="s">
+        <v>127</v>
+      </c>
+      <c r="C69" t="s">
         <v>138</v>
-      </c>
-      <c r="B69" t="s">
-        <v>128</v>
-      </c>
-      <c r="C69" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
@@ -1531,7 +1531,7 @@
         <v>72</v>
       </c>
       <c r="C71" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
@@ -1539,10 +1539,10 @@
         <v>37</v>
       </c>
       <c r="B72" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C72" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
@@ -1561,10 +1561,10 @@
         <v>5</v>
       </c>
       <c r="C75" t="s">
+        <v>100</v>
+      </c>
+      <c r="D75" t="s">
         <v>101</v>
-      </c>
-      <c r="D75" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
@@ -1594,10 +1594,10 @@
         <v>12</v>
       </c>
       <c r="B78" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C78" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
@@ -1605,10 +1605,10 @@
         <v>12</v>
       </c>
       <c r="B79" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C79" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
@@ -1616,10 +1616,10 @@
         <v>12</v>
       </c>
       <c r="B80" t="s">
+        <v>96</v>
+      </c>
+      <c r="C80" t="s">
         <v>97</v>
-      </c>
-      <c r="C80" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -1627,10 +1627,10 @@
         <v>12</v>
       </c>
       <c r="B81" t="s">
+        <v>98</v>
+      </c>
+      <c r="C81" t="s">
         <v>99</v>
-      </c>
-      <c r="C81" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
@@ -1682,10 +1682,10 @@
         <v>14</v>
       </c>
       <c r="B87" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C87" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.2">
@@ -1696,7 +1696,7 @@
         <v>18</v>
       </c>
       <c r="C89" t="s">
-        <v>82</v>
+        <v>155</v>
       </c>
       <c r="E89" t="s">
         <v>45</v>
@@ -1740,10 +1740,10 @@
         <v>17</v>
       </c>
       <c r="B93" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C93" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
@@ -1751,13 +1751,13 @@
         <v>38</v>
       </c>
       <c r="B95" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C95" t="s">
+        <v>85</v>
+      </c>
+      <c r="D95" t="s">
         <v>86</v>
-      </c>
-      <c r="D95" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
@@ -1765,10 +1765,10 @@
         <v>38</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C96" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.2">
@@ -1845,7 +1845,7 @@
         <v>68</v>
       </c>
       <c r="C104" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.2">
@@ -1856,7 +1856,7 @@
         <v>73</v>
       </c>
       <c r="C105" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.2">
@@ -1867,7 +1867,7 @@
         <v>74</v>
       </c>
       <c r="C106" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.2">
@@ -1875,10 +1875,10 @@
         <v>19</v>
       </c>
       <c r="B107" t="s">
+        <v>133</v>
+      </c>
+      <c r="C107" t="s">
         <v>134</v>
-      </c>
-      <c r="C107" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
@@ -1886,10 +1886,10 @@
         <v>19</v>
       </c>
       <c r="B108" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C108" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.2">
@@ -1897,10 +1897,10 @@
         <v>19</v>
       </c>
       <c r="B109" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C109" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.2">
@@ -1908,10 +1908,10 @@
         <v>19</v>
       </c>
       <c r="B110" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C110" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.2">
@@ -1919,10 +1919,10 @@
         <v>19</v>
       </c>
       <c r="B111" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C111" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.2">
@@ -2023,10 +2023,10 @@
         <v>20</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C122" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Minoir updates to ODM v2 general ID code
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA08EC11-9743-1947-B1CE-E055C6F6451D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68582015-AC1A-EB4A-A877-CB0BDA144D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="158">
   <si>
     <t>addresses</t>
   </si>
@@ -503,6 +503,12 @@
   </si>
   <si>
     <t>fn.makeid(datEmpty.qualityReports.qualityFlag, datEmpty.qualityReports.measureRepID, datEmpty.qualityReports.sampleID, datEmpty.qualityReports.measureSetRepID)</t>
+  </si>
+  <si>
+    <t>calculationID</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.calculations.name[:3], datEmpty.calculations.calcType[:3], datEmpty.calculations.standard)</t>
   </si>
 </sst>
 </file>
@@ -870,7 +876,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A1991E-0020-B448-B50F-72C1AC9C88C8}">
-  <dimension ref="A1:E126"/>
+  <dimension ref="A1:E127"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -968,24 +974,21 @@
         <v>140</v>
       </c>
       <c r="B9" t="s">
+        <v>156</v>
+      </c>
+      <c r="C9" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>140</v>
+      </c>
+      <c r="B10" t="s">
         <v>127</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C10" t="s">
         <v>141</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" t="s">
-        <v>103</v>
-      </c>
-      <c r="D11" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -993,45 +996,51 @@
         <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>47</v>
+        <v>103</v>
+      </c>
+      <c r="D12" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>127</v>
+      <c r="B13" t="s">
+        <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>153</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>24</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C14" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" t="s">
         <v>102</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C15" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>26</v>
-      </c>
-      <c r="B18" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1039,30 +1048,30 @@
         <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>2</v>
-      </c>
-      <c r="C19" t="s">
-        <v>83</v>
-      </c>
-      <c r="D19" t="s">
-        <v>84</v>
-      </c>
-      <c r="E19" s="1"/>
+        <v>27</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>26</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C20" t="s">
+        <v>83</v>
+      </c>
+      <c r="D20" t="s">
+        <v>84</v>
+      </c>
+      <c r="E20" s="1"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -1070,7 +1079,7 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -1078,21 +1087,18 @@
         <v>26</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>121</v>
+      <c r="B24" t="s">
+        <v>31</v>
       </c>
       <c r="C24" t="s">
-        <v>122</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
@@ -1100,242 +1106,236 @@
         <v>26</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C25" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C26" t="s">
         <v>148</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>32</v>
-      </c>
-      <c r="B27" t="s">
-        <v>16</v>
-      </c>
-      <c r="C27" t="s">
-        <v>78</v>
-      </c>
-      <c r="D27" t="s">
-        <v>59</v>
-      </c>
-      <c r="E27" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" t="s">
+        <v>78</v>
+      </c>
+      <c r="D28" t="s">
+        <v>59</v>
+      </c>
+      <c r="E28" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>32</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C29" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>3</v>
-      </c>
-      <c r="B32" t="s">
-        <v>4</v>
-      </c>
-      <c r="C32" t="s">
-        <v>79</v>
-      </c>
-      <c r="D32" t="s">
-        <v>60</v>
-      </c>
-      <c r="E32" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C33" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+      <c r="D33" t="s">
+        <v>60</v>
+      </c>
+      <c r="E33" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C34" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>3</v>
       </c>
       <c r="B35" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C35" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C36" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>3</v>
       </c>
       <c r="B37" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C37" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>3</v>
       </c>
       <c r="B38" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C38" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>3</v>
       </c>
       <c r="B39" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C39" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>3</v>
       </c>
       <c r="B40" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>3</v>
       </c>
       <c r="B41" t="s">
-        <v>109</v>
+        <v>11</v>
       </c>
       <c r="C41" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>3</v>
       </c>
       <c r="B42" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C42" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>3</v>
       </c>
       <c r="B43" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C43" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>3</v>
       </c>
       <c r="B44" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C44" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>3</v>
       </c>
       <c r="B45" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C45" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>3</v>
       </c>
       <c r="B46" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C46" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>3</v>
       </c>
       <c r="B47" t="s">
+        <v>119</v>
+      </c>
+      <c r="C47" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>3</v>
+      </c>
+      <c r="B48" t="s">
         <v>127</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C48" t="s">
         <v>128</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>34</v>
-      </c>
-      <c r="B49" t="s">
-        <v>9</v>
-      </c>
-      <c r="C49" t="s">
-        <v>94</v>
-      </c>
-      <c r="D49" t="s">
-        <v>95</v>
-      </c>
-      <c r="E49" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1343,10 +1343,16 @@
         <v>34</v>
       </c>
       <c r="B50" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C50" t="s">
-        <v>49</v>
+        <v>94</v>
+      </c>
+      <c r="D50" t="s">
+        <v>95</v>
+      </c>
+      <c r="E50" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1354,10 +1360,10 @@
         <v>34</v>
       </c>
       <c r="B51" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C51" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
@@ -1365,46 +1371,43 @@
         <v>34</v>
       </c>
       <c r="B52" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C52" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>34</v>
       </c>
-      <c r="B53" s="2" t="s">
-        <v>127</v>
+      <c r="B53" t="s">
+        <v>11</v>
       </c>
       <c r="C53" t="s">
-        <v>154</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>34</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C54" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>34</v>
+      </c>
+      <c r="B55" t="s">
         <v>93</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C55" t="s">
         <v>92</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>35</v>
-      </c>
-      <c r="B56" t="s">
-        <v>10</v>
-      </c>
-      <c r="C56" t="s">
-        <v>80</v>
-      </c>
-      <c r="D56" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
@@ -1412,10 +1415,13 @@
         <v>35</v>
       </c>
       <c r="B57" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C57" t="s">
-        <v>54</v>
+        <v>80</v>
+      </c>
+      <c r="D57" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -1423,21 +1429,21 @@
         <v>35</v>
       </c>
       <c r="B58" t="s">
+        <v>1</v>
+      </c>
+      <c r="C58" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>35</v>
+      </c>
+      <c r="B59" t="s">
         <v>127</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C59" t="s">
         <v>139</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>142</v>
-      </c>
-      <c r="B60" t="s">
-        <v>143</v>
-      </c>
-      <c r="C60" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
@@ -1445,27 +1451,21 @@
         <v>142</v>
       </c>
       <c r="B61" t="s">
+        <v>143</v>
+      </c>
+      <c r="C61" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>142</v>
+      </c>
+      <c r="B62" t="s">
         <v>127</v>
       </c>
-      <c r="C61" t="s">
+      <c r="C62" t="s">
         <v>145</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>36</v>
-      </c>
-      <c r="B63" t="s">
-        <v>7</v>
-      </c>
-      <c r="C63" t="s">
-        <v>81</v>
-      </c>
-      <c r="D63" t="s">
-        <v>63</v>
-      </c>
-      <c r="E63" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.2">
@@ -1473,10 +1473,16 @@
         <v>36</v>
       </c>
       <c r="B64" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C64" t="s">
-        <v>46</v>
+        <v>81</v>
+      </c>
+      <c r="D64" t="s">
+        <v>63</v>
+      </c>
+      <c r="E64" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
@@ -1484,10 +1490,10 @@
         <v>36</v>
       </c>
       <c r="B65" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C65" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
@@ -1495,10 +1501,10 @@
         <v>36</v>
       </c>
       <c r="B66" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C66" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
@@ -1506,32 +1512,32 @@
         <v>36</v>
       </c>
       <c r="B67" t="s">
+        <v>11</v>
+      </c>
+      <c r="C67" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>36</v>
+      </c>
+      <c r="B68" t="s">
         <v>127</v>
       </c>
-      <c r="C67" t="s">
+      <c r="C68" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
         <v>137</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B70" t="s">
         <v>127</v>
       </c>
-      <c r="C69" t="s">
+      <c r="C70" t="s">
         <v>138</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
-        <v>37</v>
-      </c>
-      <c r="B71" t="s">
-        <v>72</v>
-      </c>
-      <c r="C71" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
@@ -1539,18 +1545,21 @@
         <v>37</v>
       </c>
       <c r="B72" t="s">
+        <v>72</v>
+      </c>
+      <c r="C72" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>37</v>
+      </c>
+      <c r="B73" t="s">
         <v>127</v>
       </c>
-      <c r="C72" t="s">
+      <c r="C73" t="s">
         <v>132</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
-        <v>12</v>
-      </c>
-      <c r="B74" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
@@ -1558,13 +1567,7 @@
         <v>12</v>
       </c>
       <c r="B75" t="s">
-        <v>5</v>
-      </c>
-      <c r="C75" t="s">
-        <v>100</v>
-      </c>
-      <c r="D75" t="s">
-        <v>101</v>
+        <v>13</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
@@ -1572,10 +1575,13 @@
         <v>12</v>
       </c>
       <c r="B76" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C76" t="s">
-        <v>47</v>
+        <v>100</v>
+      </c>
+      <c r="D76" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
@@ -1583,10 +1589,10 @@
         <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C77" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
@@ -1594,10 +1600,10 @@
         <v>12</v>
       </c>
       <c r="B78" t="s">
-        <v>127</v>
+        <v>11</v>
       </c>
       <c r="C78" t="s">
-        <v>146</v>
+        <v>48</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
@@ -1605,10 +1611,10 @@
         <v>12</v>
       </c>
       <c r="B79" t="s">
-        <v>93</v>
+        <v>127</v>
       </c>
       <c r="C79" t="s">
-        <v>92</v>
+        <v>146</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
@@ -1616,10 +1622,10 @@
         <v>12</v>
       </c>
       <c r="B80" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C80" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -1627,21 +1633,21 @@
         <v>12</v>
       </c>
       <c r="B81" t="s">
+        <v>96</v>
+      </c>
+      <c r="C81" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>12</v>
+      </c>
+      <c r="B82" t="s">
         <v>98</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C82" t="s">
         <v>99</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>14</v>
-      </c>
-      <c r="B83" t="s">
-        <v>15</v>
-      </c>
-      <c r="C83" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
@@ -1649,10 +1655,10 @@
         <v>14</v>
       </c>
       <c r="B84" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C84" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
@@ -1660,10 +1666,10 @@
         <v>14</v>
       </c>
       <c r="B85" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C85" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.2">
@@ -1671,10 +1677,10 @@
         <v>14</v>
       </c>
       <c r="B86" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C86" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
@@ -1682,24 +1688,21 @@
         <v>14</v>
       </c>
       <c r="B87" t="s">
+        <v>16</v>
+      </c>
+      <c r="C87" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>14</v>
+      </c>
+      <c r="B88" t="s">
         <v>127</v>
       </c>
-      <c r="C87" t="s">
+      <c r="C88" t="s">
         <v>131</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
-        <v>17</v>
-      </c>
-      <c r="B89" t="s">
-        <v>18</v>
-      </c>
-      <c r="C89" t="s">
-        <v>155</v>
-      </c>
-      <c r="E89" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
@@ -1707,10 +1710,13 @@
         <v>17</v>
       </c>
       <c r="B90" t="s">
-        <v>4</v>
+        <v>18</v>
+      </c>
+      <c r="C90" t="s">
+        <v>155</v>
       </c>
       <c r="E90" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
@@ -1718,10 +1724,10 @@
         <v>17</v>
       </c>
       <c r="B91" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E91" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
@@ -1729,10 +1735,10 @@
         <v>17</v>
       </c>
       <c r="B92" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E92" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
@@ -1740,49 +1746,46 @@
         <v>17</v>
       </c>
       <c r="B93" t="s">
+        <v>9</v>
+      </c>
+      <c r="E93" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>17</v>
+      </c>
+      <c r="B94" t="s">
         <v>127</v>
       </c>
-      <c r="C93" t="s">
+      <c r="C94" t="s">
         <v>129</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
-        <v>38</v>
-      </c>
-      <c r="B95" t="s">
-        <v>87</v>
-      </c>
-      <c r="C95" t="s">
-        <v>85</v>
-      </c>
-      <c r="D95" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>38</v>
       </c>
-      <c r="B96" s="2" t="s">
+      <c r="B96" t="s">
+        <v>87</v>
+      </c>
+      <c r="C96" t="s">
+        <v>85</v>
+      </c>
+      <c r="D96" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>38</v>
+      </c>
+      <c r="B97" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C96" t="s">
+      <c r="C97" t="s">
         <v>150</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
-        <v>19</v>
-      </c>
-      <c r="B98" t="s">
-        <v>6</v>
-      </c>
-      <c r="C98" t="s">
-        <v>76</v>
-      </c>
-      <c r="D98" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
@@ -1790,7 +1793,13 @@
         <v>19</v>
       </c>
       <c r="B99" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="C99" t="s">
+        <v>76</v>
+      </c>
+      <c r="D99" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.2">
@@ -1798,10 +1807,7 @@
         <v>19</v>
       </c>
       <c r="B100" t="s">
-        <v>10</v>
-      </c>
-      <c r="C100" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.2">
@@ -1809,10 +1815,10 @@
         <v>19</v>
       </c>
       <c r="B101" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C101" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.2">
@@ -1820,10 +1826,10 @@
         <v>19</v>
       </c>
       <c r="B102" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C102" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.2">
@@ -1831,10 +1837,10 @@
         <v>19</v>
       </c>
       <c r="B103" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C103" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.2">
@@ -1842,10 +1848,10 @@
         <v>19</v>
       </c>
       <c r="B104" t="s">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="C104" t="s">
-        <v>106</v>
+        <v>46</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.2">
@@ -1853,10 +1859,10 @@
         <v>19</v>
       </c>
       <c r="B105" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C105" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.2">
@@ -1864,10 +1870,10 @@
         <v>19</v>
       </c>
       <c r="B106" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C106" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.2">
@@ -1875,10 +1881,10 @@
         <v>19</v>
       </c>
       <c r="B107" t="s">
-        <v>133</v>
+        <v>74</v>
       </c>
       <c r="C107" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
@@ -1886,10 +1892,10 @@
         <v>19</v>
       </c>
       <c r="B108" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="C108" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.2">
@@ -1897,10 +1903,10 @@
         <v>19</v>
       </c>
       <c r="B109" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C109" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.2">
@@ -1908,10 +1914,10 @@
         <v>19</v>
       </c>
       <c r="B110" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="C110" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.2">
@@ -1919,18 +1925,21 @@
         <v>19</v>
       </c>
       <c r="B111" t="s">
+        <v>119</v>
+      </c>
+      <c r="C111" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>19</v>
+      </c>
+      <c r="B112" t="s">
         <v>127</v>
       </c>
-      <c r="C111" t="s">
+      <c r="C112" t="s">
         <v>136</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A113" t="s">
-        <v>20</v>
-      </c>
-      <c r="B113" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.2">
@@ -1938,13 +1947,7 @@
         <v>20</v>
       </c>
       <c r="B114" t="s">
-        <v>8</v>
-      </c>
-      <c r="C114" t="s">
-        <v>75</v>
-      </c>
-      <c r="D114" t="s">
-        <v>64</v>
+        <v>21</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.2">
@@ -1952,10 +1955,13 @@
         <v>20</v>
       </c>
       <c r="B115" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C115" t="s">
-        <v>46</v>
+        <v>75</v>
+      </c>
+      <c r="D115" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.2">
@@ -1963,10 +1969,10 @@
         <v>20</v>
       </c>
       <c r="B116" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C116" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.2">
@@ -1974,10 +1980,10 @@
         <v>20</v>
       </c>
       <c r="B117" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C117" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.2">
@@ -1985,10 +1991,10 @@
         <v>20</v>
       </c>
       <c r="B118" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C118" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.2">
@@ -1996,10 +2002,10 @@
         <v>20</v>
       </c>
       <c r="B119" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C119" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.2">
@@ -2007,7 +2013,10 @@
         <v>20</v>
       </c>
       <c r="B120" t="s">
-        <v>22</v>
+        <v>11</v>
+      </c>
+      <c r="C120" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.2">
@@ -2015,27 +2024,35 @@
         <v>20</v>
       </c>
       <c r="B121" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>20</v>
       </c>
-      <c r="B122" s="2" t="s">
+      <c r="B122" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A123" t="s">
+        <v>20</v>
+      </c>
+      <c r="B123" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C122" t="s">
+      <c r="C123" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A124" t="s">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A126" t="s">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
For primary key IDs that have already been populated (before ID generation), use the original ID unchanged (previously they were being formatted with fn.makeid)
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68582015-AC1A-EB4A-A877-CB0BDA144D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110586EA-0730-234C-86CF-FFF5857DE6E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -262,39 +262,12 @@
     <t>collDTEnd</t>
   </si>
   <si>
-    <t>fn.makeid(dat.sites.__siteID)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.samples.__sampleID)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.addresses.__addressID)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.instruments.__instrumentID)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.measures.__measureRepID)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.organizations.__organizationID)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.polygons.__polygonID)</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.protocolRelationships.protocolIDContainer, datEmpty.protocolRelationships.stepIDObj, datEmpty.protocolRelationships.relationshipID)</t>
   </si>
   <si>
-    <t>fn.makeid(dat.datasets.__datasetID)</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.organizations.organizationID)</t>
   </si>
   <si>
-    <t>fn.makeid(dat.sampleRelationships.__sampleRelationshipsID)</t>
-  </si>
-  <si>
     <t>fn.makeid("rel")</t>
   </si>
   <si>
@@ -307,9 +280,6 @@
     <t>accessIndexID</t>
   </si>
   <si>
-    <t>fn.makeid(dat.accessions.__accessIndexID)</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.accessions.organizationID, datEmpty.accessions.dataHost, datEmpty.accessions.accessNum)</t>
   </si>
   <si>
@@ -319,9 +289,6 @@
     <t>_extra_measures_count</t>
   </si>
   <si>
-    <t>fn.makeid(dat.measures.__measureSetRepID) if int(dat.measureSets._extra_measures_count) else ""</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(int(dat.measureSets._extra_measures_count))) if int(dat.measureSets._extra_measures_count) else ""</t>
   </si>
   <si>
@@ -337,18 +304,12 @@
     <t>int(dat.protocols._extra_measures_count) + int(dat.protocols._extra_protocolSteps_count)</t>
   </si>
   <si>
-    <t>fn.makeid(dat.protocols.__protocolID) if int(dat.protocols._extra_fk_count) else ""</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.protocols.name, datEmpty.protocols.protocolVersion) if int(dat.protocols._extra_fk_count) else ""</t>
   </si>
   <si>
     <t>_extra_has_data</t>
   </si>
   <si>
-    <t>fn.makeid(dat.contacts.__contactID) if dat.contacts._extra_has_data else ""</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.organizations.organizationID, datEmpty.contacts.role[:3]) if dat.contacts._extra_has_data else ""</t>
   </si>
   <si>
@@ -509,6 +470,45 @@
   </si>
   <si>
     <t>fn.makeid(datEmpty.calculations.name[:3], datEmpty.calculations.calcType[:3], datEmpty.calculations.standard)</t>
+  </si>
+  <si>
+    <t>dat.accessions.__accessIndexID</t>
+  </si>
+  <si>
+    <t>dat.addresses.__addressID</t>
+  </si>
+  <si>
+    <t>dat.contacts.__contactID if dat.contacts._extra_has_data else ""</t>
+  </si>
+  <si>
+    <t>dat.datasets.__datasetID</t>
+  </si>
+  <si>
+    <t>dat.instruments.__instrumentID</t>
+  </si>
+  <si>
+    <t>dat.measures.__measureRepID</t>
+  </si>
+  <si>
+    <t>dat.measures.__measureSetRepID if int(dat.measureSets._extra_measures_count) else ""</t>
+  </si>
+  <si>
+    <t>dat.organizations.__organizationID</t>
+  </si>
+  <si>
+    <t>dat.polygons.__polygonID</t>
+  </si>
+  <si>
+    <t>dat.protocols.__protocolID if int(dat.protocols._extra_fk_count) else ""</t>
+  </si>
+  <si>
+    <t>dat.sampleRelationships.__sampleRelationshipsID</t>
+  </si>
+  <si>
+    <t>dat.samples.__sampleID</t>
+  </si>
+  <si>
+    <t>dat.sites.__siteID</t>
   </si>
 </sst>
 </file>
@@ -901,21 +901,21 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B2" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
-        <v>90</v>
+        <v>145</v>
       </c>
       <c r="D2" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
@@ -926,13 +926,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B4" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C4" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -949,7 +949,7 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>77</v>
+        <v>146</v>
       </c>
       <c r="D6" t="s">
         <v>71</v>
@@ -963,32 +963,32 @@
         <v>0</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C7" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="B9" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
       <c r="C9" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="B10" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C10" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -999,10 +999,10 @@
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>103</v>
+        <v>147</v>
       </c>
       <c r="D12" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -1021,10 +1021,10 @@
         <v>24</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C14" t="s">
-        <v>153</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -1032,10 +1032,10 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="C15" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -1059,10 +1059,10 @@
         <v>2</v>
       </c>
       <c r="C20" t="s">
-        <v>83</v>
+        <v>148</v>
       </c>
       <c r="D20" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="E20" s="1"/>
     </row>
@@ -1106,10 +1106,10 @@
         <v>26</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="C25" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -1117,10 +1117,10 @@
         <v>26</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C26" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -1131,7 +1131,7 @@
         <v>16</v>
       </c>
       <c r="C28" t="s">
-        <v>78</v>
+        <v>149</v>
       </c>
       <c r="D28" t="s">
         <v>59</v>
@@ -1145,10 +1145,10 @@
         <v>32</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C29" t="s">
-        <v>151</v>
+        <v>138</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1164,7 +1164,7 @@
         <v>4</v>
       </c>
       <c r="C33" t="s">
-        <v>79</v>
+        <v>150</v>
       </c>
       <c r="D33" t="s">
         <v>60</v>
@@ -1266,10 +1266,10 @@
         <v>3</v>
       </c>
       <c r="B42" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="C42" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
@@ -1277,10 +1277,10 @@
         <v>3</v>
       </c>
       <c r="B43" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="C43" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
@@ -1288,10 +1288,10 @@
         <v>3</v>
       </c>
       <c r="B44" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="C44" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -1299,10 +1299,10 @@
         <v>3</v>
       </c>
       <c r="B45" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="C45" t="s">
-        <v>117</v>
+        <v>104</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
@@ -1310,10 +1310,10 @@
         <v>3</v>
       </c>
       <c r="B46" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="C46" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -1321,10 +1321,10 @@
         <v>3</v>
       </c>
       <c r="B47" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="C47" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -1332,10 +1332,10 @@
         <v>3</v>
       </c>
       <c r="B48" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C48" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1346,10 +1346,10 @@
         <v>9</v>
       </c>
       <c r="C50" t="s">
-        <v>94</v>
+        <v>151</v>
       </c>
       <c r="D50" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="E50" t="s">
         <v>61</v>
@@ -1393,10 +1393,10 @@
         <v>34</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C54" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
@@ -1404,10 +1404,10 @@
         <v>34</v>
       </c>
       <c r="B55" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="C55" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
@@ -1418,7 +1418,7 @@
         <v>10</v>
       </c>
       <c r="C57" t="s">
-        <v>80</v>
+        <v>152</v>
       </c>
       <c r="D57" t="s">
         <v>62</v>
@@ -1440,32 +1440,32 @@
         <v>35</v>
       </c>
       <c r="B59" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C59" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="B61" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="C61" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="B62" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C62" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.2">
@@ -1476,7 +1476,7 @@
         <v>7</v>
       </c>
       <c r="C64" t="s">
-        <v>81</v>
+        <v>153</v>
       </c>
       <c r="D64" t="s">
         <v>63</v>
@@ -1523,21 +1523,21 @@
         <v>36</v>
       </c>
       <c r="B68" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C68" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="B70" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C70" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
@@ -1548,7 +1548,7 @@
         <v>72</v>
       </c>
       <c r="C72" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
@@ -1556,10 +1556,10 @@
         <v>37</v>
       </c>
       <c r="B73" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C73" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
@@ -1578,10 +1578,10 @@
         <v>5</v>
       </c>
       <c r="C76" t="s">
-        <v>100</v>
+        <v>154</v>
       </c>
       <c r="D76" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
@@ -1611,10 +1611,10 @@
         <v>12</v>
       </c>
       <c r="B79" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C79" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
@@ -1622,10 +1622,10 @@
         <v>12</v>
       </c>
       <c r="B80" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="C80" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -1633,10 +1633,10 @@
         <v>12</v>
       </c>
       <c r="B81" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="C81" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
@@ -1644,10 +1644,10 @@
         <v>12</v>
       </c>
       <c r="B82" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C82" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
@@ -1699,10 +1699,10 @@
         <v>14</v>
       </c>
       <c r="B88" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C88" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
@@ -1713,7 +1713,7 @@
         <v>18</v>
       </c>
       <c r="C90" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="E90" t="s">
         <v>45</v>
@@ -1757,10 +1757,10 @@
         <v>17</v>
       </c>
       <c r="B94" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C94" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
@@ -1768,13 +1768,13 @@
         <v>38</v>
       </c>
       <c r="B96" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="C96" t="s">
-        <v>85</v>
+        <v>155</v>
       </c>
       <c r="D96" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
@@ -1782,10 +1782,10 @@
         <v>38</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C97" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
@@ -1796,7 +1796,7 @@
         <v>6</v>
       </c>
       <c r="C99" t="s">
-        <v>76</v>
+        <v>156</v>
       </c>
       <c r="D99" t="s">
         <v>70</v>
@@ -1862,7 +1862,7 @@
         <v>68</v>
       </c>
       <c r="C105" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.2">
@@ -1873,7 +1873,7 @@
         <v>73</v>
       </c>
       <c r="C106" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.2">
@@ -1884,7 +1884,7 @@
         <v>74</v>
       </c>
       <c r="C107" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
@@ -1892,10 +1892,10 @@
         <v>19</v>
       </c>
       <c r="B108" t="s">
-        <v>133</v>
+        <v>120</v>
       </c>
       <c r="C108" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.2">
@@ -1903,10 +1903,10 @@
         <v>19</v>
       </c>
       <c r="B109" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="C109" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.2">
@@ -1914,10 +1914,10 @@
         <v>19</v>
       </c>
       <c r="B110" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="C110" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.2">
@@ -1925,10 +1925,10 @@
         <v>19</v>
       </c>
       <c r="B111" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="C111" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.2">
@@ -1936,10 +1936,10 @@
         <v>19</v>
       </c>
       <c r="B112" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C112" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.2">
@@ -1958,7 +1958,7 @@
         <v>8</v>
       </c>
       <c r="C115" t="s">
-        <v>75</v>
+        <v>157</v>
       </c>
       <c r="D115" t="s">
         <v>64</v>
@@ -2040,10 +2040,10 @@
         <v>20</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C123" t="s">
-        <v>152</v>
+        <v>139</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Changed all primary keys to be passed to fn.makeid
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110586EA-0730-234C-86CF-FFF5857DE6E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CEAE782-4BF4-314E-9910-0CE33C9C0372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -268,9 +268,6 @@
     <t>fn.makeid(datEmpty.organizations.organizationID)</t>
   </si>
   <si>
-    <t>fn.makeid("rel")</t>
-  </si>
-  <si>
     <t>sampleRelationshipsID</t>
   </si>
   <si>
@@ -472,43 +469,46 @@
     <t>fn.makeid(datEmpty.calculations.name[:3], datEmpty.calculations.calcType[:3], datEmpty.calculations.standard)</t>
   </si>
   <si>
-    <t>dat.accessions.__accessIndexID</t>
-  </si>
-  <si>
-    <t>dat.addresses.__addressID</t>
-  </si>
-  <si>
-    <t>dat.contacts.__contactID if dat.contacts._extra_has_data else ""</t>
-  </si>
-  <si>
-    <t>dat.datasets.__datasetID</t>
-  </si>
-  <si>
-    <t>dat.instruments.__instrumentID</t>
-  </si>
-  <si>
-    <t>dat.measures.__measureRepID</t>
-  </si>
-  <si>
-    <t>dat.measures.__measureSetRepID if int(dat.measureSets._extra_measures_count) else ""</t>
-  </si>
-  <si>
-    <t>dat.organizations.__organizationID</t>
-  </si>
-  <si>
-    <t>dat.polygons.__polygonID</t>
-  </si>
-  <si>
-    <t>dat.protocols.__protocolID if int(dat.protocols._extra_fk_count) else ""</t>
-  </si>
-  <si>
-    <t>dat.sampleRelationships.__sampleRelationshipsID</t>
-  </si>
-  <si>
-    <t>dat.samples.__sampleID</t>
-  </si>
-  <si>
-    <t>dat.sites.__siteID</t>
+    <t>fn.makeid(dat.protocols.__protocolID) if int(dat.protocols._extra_fk_count) else ""</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.accessions.__accessIndexID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.addresses.__addressID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.contacts.__contactID) if dat.contacts._extra_has_data else ""</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.datasets.__datasetID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.instruments.__instrumentID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.measures.__measureRepID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.measures.__measureSetRepID) if int(dat.measureSets._extra_measures_count) else ""</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.organizations.__organizationID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.polygons.__polygonID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.sampleRelationships.__sampleRelationshipsID)</t>
+  </si>
+  <si>
+    <t>fn.makeid("sar")</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.samples.__sampleID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.sites.__siteID)</t>
   </si>
 </sst>
 </file>
@@ -901,21 +901,21 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" t="s">
         <v>79</v>
-      </c>
-      <c r="B2" t="s">
-        <v>80</v>
       </c>
       <c r="C2" t="s">
         <v>145</v>
       </c>
       <c r="D2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
@@ -926,13 +926,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -963,32 +963,32 @@
         <v>0</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C9" t="s">
         <v>143</v>
-      </c>
-      <c r="C9" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" t="s">
         <v>127</v>
-      </c>
-      <c r="B10" t="s">
-        <v>114</v>
-      </c>
-      <c r="C10" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -1002,7 +1002,7 @@
         <v>147</v>
       </c>
       <c r="D12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -1021,10 +1021,10 @@
         <v>24</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -1032,10 +1032,10 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -1106,10 +1106,10 @@
         <v>26</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C25" t="s">
         <v>108</v>
-      </c>
-      <c r="C25" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -1117,10 +1117,10 @@
         <v>26</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C26" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -1145,10 +1145,10 @@
         <v>32</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C29" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1266,10 +1266,10 @@
         <v>3</v>
       </c>
       <c r="B42" t="s">
+        <v>95</v>
+      </c>
+      <c r="C42" t="s">
         <v>96</v>
-      </c>
-      <c r="C42" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
@@ -1277,10 +1277,10 @@
         <v>3</v>
       </c>
       <c r="B43" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C43" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
@@ -1288,10 +1288,10 @@
         <v>3</v>
       </c>
       <c r="B44" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C44" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -1299,10 +1299,10 @@
         <v>3</v>
       </c>
       <c r="B45" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C45" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
@@ -1310,10 +1310,10 @@
         <v>3</v>
       </c>
       <c r="B46" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C46" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -1321,10 +1321,10 @@
         <v>3</v>
       </c>
       <c r="B47" t="s">
+        <v>105</v>
+      </c>
+      <c r="C47" t="s">
         <v>106</v>
-      </c>
-      <c r="C47" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -1332,10 +1332,10 @@
         <v>3</v>
       </c>
       <c r="B48" t="s">
+        <v>113</v>
+      </c>
+      <c r="C48" t="s">
         <v>114</v>
-      </c>
-      <c r="C48" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1349,7 +1349,7 @@
         <v>151</v>
       </c>
       <c r="D50" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E50" t="s">
         <v>61</v>
@@ -1393,10 +1393,10 @@
         <v>34</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C54" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
@@ -1404,10 +1404,10 @@
         <v>34</v>
       </c>
       <c r="B55" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C55" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
@@ -1440,32 +1440,32 @@
         <v>35</v>
       </c>
       <c r="B59" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C59" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
+        <v>128</v>
+      </c>
+      <c r="B61" t="s">
         <v>129</v>
       </c>
-      <c r="B61" t="s">
+      <c r="C61" t="s">
         <v>130</v>
-      </c>
-      <c r="C61" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B62" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C62" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.2">
@@ -1523,21 +1523,21 @@
         <v>36</v>
       </c>
       <c r="B68" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C68" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
+        <v>123</v>
+      </c>
+      <c r="B70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C70" t="s">
         <v>124</v>
-      </c>
-      <c r="B70" t="s">
-        <v>114</v>
-      </c>
-      <c r="C70" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
@@ -1556,10 +1556,10 @@
         <v>37</v>
       </c>
       <c r="B73" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C73" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
@@ -1578,10 +1578,10 @@
         <v>5</v>
       </c>
       <c r="C76" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="D76" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
@@ -1611,10 +1611,10 @@
         <v>12</v>
       </c>
       <c r="B79" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C79" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
@@ -1622,10 +1622,10 @@
         <v>12</v>
       </c>
       <c r="B80" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C80" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -1633,10 +1633,10 @@
         <v>12</v>
       </c>
       <c r="B81" t="s">
+        <v>84</v>
+      </c>
+      <c r="C81" t="s">
         <v>85</v>
-      </c>
-      <c r="C81" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
@@ -1644,10 +1644,10 @@
         <v>12</v>
       </c>
       <c r="B82" t="s">
+        <v>86</v>
+      </c>
+      <c r="C82" t="s">
         <v>87</v>
-      </c>
-      <c r="C82" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
@@ -1699,10 +1699,10 @@
         <v>14</v>
       </c>
       <c r="B88" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C88" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
@@ -1713,7 +1713,7 @@
         <v>18</v>
       </c>
       <c r="C90" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E90" t="s">
         <v>45</v>
@@ -1757,10 +1757,10 @@
         <v>17</v>
       </c>
       <c r="B94" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C94" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
@@ -1768,13 +1768,13 @@
         <v>38</v>
       </c>
       <c r="B96" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C96" t="s">
+        <v>154</v>
+      </c>
+      <c r="D96" t="s">
         <v>155</v>
-      </c>
-      <c r="D96" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
@@ -1782,10 +1782,10 @@
         <v>38</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C97" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
@@ -1862,7 +1862,7 @@
         <v>68</v>
       </c>
       <c r="C105" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.2">
@@ -1873,7 +1873,7 @@
         <v>73</v>
       </c>
       <c r="C106" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.2">
@@ -1884,7 +1884,7 @@
         <v>74</v>
       </c>
       <c r="C107" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
@@ -1892,10 +1892,10 @@
         <v>19</v>
       </c>
       <c r="B108" t="s">
+        <v>119</v>
+      </c>
+      <c r="C108" t="s">
         <v>120</v>
-      </c>
-      <c r="C108" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.2">
@@ -1903,10 +1903,10 @@
         <v>19</v>
       </c>
       <c r="B109" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C109" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.2">
@@ -1914,10 +1914,10 @@
         <v>19</v>
       </c>
       <c r="B110" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C110" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.2">
@@ -1925,10 +1925,10 @@
         <v>19</v>
       </c>
       <c r="B111" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C111" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.2">
@@ -1936,10 +1936,10 @@
         <v>19</v>
       </c>
       <c r="B112" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C112" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.2">
@@ -2040,10 +2040,10 @@
         <v>20</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C123" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
- Remove "emap" namespace use (for compatibility with new linkml-map) in mapper YAMLs. - Replace "".format(...) with "%d" % (...) for ID generation in general_v2_id_code.xlsx. - Add "range: Any" for slots that use any_of (convention used by latest linkml) in pha4ge.yaml. - Add try block for permissible_value_ancestors call (new linkml raises an exception for unrecognized ranges) in enum_hierarchy_selector.py.
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/_shared/ids/general_v2_id_code.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/_shared/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CEAE782-4BF4-314E-9910-0CE33C9C0372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FFC2DBA-AE0D-1B48-BE05-9EBCE4B4EB92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="40960" windowHeight="20760" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
   <sheets>
     <sheet name="id_code" sheetId="1" r:id="rId1"/>
@@ -220,9 +220,6 @@
     <t>fn.makeid(datEmpty.measures.sampleID, datEmpty.measures.measure)</t>
   </si>
   <si>
-    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures", "__measureSetRepID", equals=datEmpty.measureSets.__measureSetRepID)))</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.addresses.addressID, datEmpty.organizations.name[:3])</t>
   </si>
   <si>
@@ -286,9 +283,6 @@
     <t>_extra_measures_count</t>
   </si>
   <si>
-    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(int(dat.measureSets._extra_measures_count))) if int(dat.measureSets._extra_measures_count) else ""</t>
-  </si>
-  <si>
     <t>_extra_protocolSteps_count</t>
   </si>
   <si>
@@ -509,6 +503,12 @@
   </si>
   <si>
     <t>fn.makeid(dat.sites.__siteID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.measures.measureRepID, "%04d" % (int(dat.measureSets._extra_measures_count))) if int(dat.measureSets._extra_measures_count) else ""</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.measures.measureRepID, "%04d" % (fn.countrows("measures", "__measureSetRepID", equals=datEmpty.measureSets.__measureSetRepID)))</t>
   </si>
 </sst>
 </file>
@@ -901,21 +901,21 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" t="s">
         <v>78</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" t="s">
         <v>79</v>
-      </c>
-      <c r="C2" t="s">
-        <v>145</v>
-      </c>
-      <c r="D2" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
@@ -926,13 +926,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -949,13 +949,13 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -963,32 +963,32 @@
         <v>0</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B9" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C9" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -999,10 +999,10 @@
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D12" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -1021,10 +1021,10 @@
         <v>24</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C14" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -1032,10 +1032,10 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
+        <v>87</v>
+      </c>
+      <c r="C15" t="s">
         <v>89</v>
-      </c>
-      <c r="C15" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -1059,10 +1059,10 @@
         <v>2</v>
       </c>
       <c r="C20" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E20" s="1"/>
     </row>
@@ -1106,10 +1106,10 @@
         <v>26</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C25" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -1117,10 +1117,10 @@
         <v>26</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C26" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -1131,13 +1131,13 @@
         <v>16</v>
       </c>
       <c r="C28" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D28" t="s">
         <v>59</v>
       </c>
       <c r="E28" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -1145,10 +1145,10 @@
         <v>32</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C29" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1164,13 +1164,13 @@
         <v>4</v>
       </c>
       <c r="C33" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D33" t="s">
         <v>60</v>
       </c>
       <c r="E33" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
@@ -1266,10 +1266,10 @@
         <v>3</v>
       </c>
       <c r="B42" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C42" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
@@ -1277,10 +1277,10 @@
         <v>3</v>
       </c>
       <c r="B43" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C43" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
@@ -1288,10 +1288,10 @@
         <v>3</v>
       </c>
       <c r="B44" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C44" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -1299,10 +1299,10 @@
         <v>3</v>
       </c>
       <c r="B45" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C45" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
@@ -1310,10 +1310,10 @@
         <v>3</v>
       </c>
       <c r="B46" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C46" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -1321,10 +1321,10 @@
         <v>3</v>
       </c>
       <c r="B47" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C47" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -1332,10 +1332,10 @@
         <v>3</v>
       </c>
       <c r="B48" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C48" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1346,13 +1346,13 @@
         <v>9</v>
       </c>
       <c r="C50" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D50" t="s">
-        <v>83</v>
+        <v>156</v>
       </c>
       <c r="E50" t="s">
-        <v>61</v>
+        <v>157</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1393,10 +1393,10 @@
         <v>34</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C54" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
@@ -1404,10 +1404,10 @@
         <v>34</v>
       </c>
       <c r="B55" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C55" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
@@ -1418,10 +1418,10 @@
         <v>10</v>
       </c>
       <c r="C57" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D57" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -1440,32 +1440,32 @@
         <v>35</v>
       </c>
       <c r="B59" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C59" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
+        <v>126</v>
+      </c>
+      <c r="B61" t="s">
+        <v>127</v>
+      </c>
+      <c r="C61" t="s">
         <v>128</v>
-      </c>
-      <c r="B61" t="s">
-        <v>129</v>
-      </c>
-      <c r="C61" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B62" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C62" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.2">
@@ -1476,13 +1476,13 @@
         <v>7</v>
       </c>
       <c r="C64" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D64" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E64" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
@@ -1523,21 +1523,21 @@
         <v>36</v>
       </c>
       <c r="B68" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C68" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B70" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C70" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
@@ -1545,10 +1545,10 @@
         <v>37</v>
       </c>
       <c r="B72" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C72" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
@@ -1556,10 +1556,10 @@
         <v>37</v>
       </c>
       <c r="B73" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C73" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
@@ -1578,10 +1578,10 @@
         <v>5</v>
       </c>
       <c r="C76" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D76" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
@@ -1611,10 +1611,10 @@
         <v>12</v>
       </c>
       <c r="B79" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C79" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
@@ -1622,10 +1622,10 @@
         <v>12</v>
       </c>
       <c r="B80" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C80" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -1633,10 +1633,10 @@
         <v>12</v>
       </c>
       <c r="B81" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C81" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
@@ -1644,10 +1644,10 @@
         <v>12</v>
       </c>
       <c r="B82" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C82" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
@@ -1658,7 +1658,7 @@
         <v>15</v>
       </c>
       <c r="C84" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
@@ -1699,10 +1699,10 @@
         <v>14</v>
       </c>
       <c r="B88" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C88" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
@@ -1713,7 +1713,7 @@
         <v>18</v>
       </c>
       <c r="C90" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E90" t="s">
         <v>45</v>
@@ -1757,10 +1757,10 @@
         <v>17</v>
       </c>
       <c r="B94" t="s">
+        <v>111</v>
+      </c>
+      <c r="C94" t="s">
         <v>113</v>
-      </c>
-      <c r="C94" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
@@ -1768,13 +1768,13 @@
         <v>38</v>
       </c>
       <c r="B96" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C96" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D96" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
@@ -1782,10 +1782,10 @@
         <v>38</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C97" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
@@ -1796,10 +1796,10 @@
         <v>6</v>
       </c>
       <c r="C99" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D99" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.2">
@@ -1859,10 +1859,10 @@
         <v>19</v>
       </c>
       <c r="B105" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C105" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.2">
@@ -1870,10 +1870,10 @@
         <v>19</v>
       </c>
       <c r="B106" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C106" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.2">
@@ -1881,10 +1881,10 @@
         <v>19</v>
       </c>
       <c r="B107" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C107" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
@@ -1892,10 +1892,10 @@
         <v>19</v>
       </c>
       <c r="B108" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C108" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.2">
@@ -1903,10 +1903,10 @@
         <v>19</v>
       </c>
       <c r="B109" t="s">
+        <v>107</v>
+      </c>
+      <c r="C109" t="s">
         <v>109</v>
-      </c>
-      <c r="C109" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.2">
@@ -1914,10 +1914,10 @@
         <v>19</v>
       </c>
       <c r="B110" t="s">
+        <v>108</v>
+      </c>
+      <c r="C110" t="s">
         <v>110</v>
-      </c>
-      <c r="C110" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.2">
@@ -1925,10 +1925,10 @@
         <v>19</v>
       </c>
       <c r="B111" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C111" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.2">
@@ -1936,10 +1936,10 @@
         <v>19</v>
       </c>
       <c r="B112" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C112" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.2">
@@ -1958,10 +1958,10 @@
         <v>8</v>
       </c>
       <c r="C115" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D115" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.2">
@@ -2040,10 +2040,10 @@
         <v>20</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C123" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>